<commit_message>
Add Barra orders 106016 and 106020
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9PfgDEdKqrS7U5PG39u7r
</commit_message>
<xml_diff>
--- a/pedidos/Pedidos_Fev27_Unificado.xlsx
+++ b/pedidos/Pedidos_Fev27_Unificado.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA194"/>
+  <dimension ref="A1:AA203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12631,7 +12631,7 @@
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>106004</v>
+        <v>106020</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -12639,21 +12639,21 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>99069512</v>
+        <v>194876138</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ADP160</t>
+          <t>SSU030</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>ADP160CF</t>
+          <t>SSU030CF</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>ADP160CF</t>
+          <t>SSU030CF</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -12663,24 +12663,24 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>MOCASSIM</t>
+          <t>TENIS</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>CLASSICO</t>
+          <t>VERAO</t>
         </is>
       </c>
       <c r="J181" t="n">
-        <v>439.9</v>
+        <v>299.9</v>
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="L181" t="n">
-        <v>148.03</v>
+        <v>99.92</v>
       </c>
       <c r="M181" t="n">
         <v>1</v>
@@ -12692,30 +12692,27 @@
         <v>4</v>
       </c>
       <c r="T181" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U181" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V181" t="n">
         <v>4</v>
       </c>
       <c r="W181" t="n">
-        <v>3</v>
-      </c>
-      <c r="X181" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z181" t="n">
         <v>24</v>
       </c>
       <c r="AA181" t="n">
-        <v>3552.72</v>
+        <v>2398.08</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>106004</v>
+        <v>106020</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -12723,21 +12720,21 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>56456539</v>
+        <v>151143141</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>ASF950</t>
+          <t>SSU030</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>ASF950TP</t>
+          <t>SSU030OW</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>ASF950TP</t>
+          <t>SSU030OW</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -12747,24 +12744,24 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>SANDALIA</t>
+          <t>TENIS</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>VERAO</t>
+          <t>INVERNO</t>
         </is>
       </c>
       <c r="J182" t="n">
-        <v>399.9</v>
+        <v>299.9</v>
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="L182" t="n">
-        <v>124.86</v>
+        <v>99.92</v>
       </c>
       <c r="M182" t="n">
         <v>1</v>
@@ -12773,33 +12770,30 @@
         <v>2</v>
       </c>
       <c r="S182" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="T182" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U182" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="V182" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W182" t="n">
-        <v>3</v>
-      </c>
-      <c r="X182" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Z182" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="AA182" t="n">
-        <v>2996.64</v>
+        <v>3597.12</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>106004</v>
+        <v>106020</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -12807,36 +12801,36 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>63032743</v>
+        <v>151143142</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>PRAD44</t>
+          <t>SSU030</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>PRAD44TP</t>
+          <t>SSU030PT</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>PRAD44TP</t>
+          <t>SSU030PT</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>FEMININO</t>
+          <t>MASCULINO</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>SANDALIA BIRKEN</t>
+          <t>TENIS</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>CLASSICO</t>
+          <t>INVERNO</t>
         </is>
       </c>
       <c r="J183" t="n">
@@ -12844,43 +12838,43 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="L183" t="n">
-        <v>119.46</v>
+        <v>99.92</v>
       </c>
       <c r="M183" t="n">
         <v>1</v>
       </c>
-      <c r="N183" t="n">
-        <v>2</v>
-      </c>
-      <c r="O183" t="n">
+      <c r="R183" t="n">
+        <v>2</v>
+      </c>
+      <c r="S183" t="n">
         <v>6</v>
       </c>
-      <c r="P183" t="n">
+      <c r="T183" t="n">
         <v>10</v>
       </c>
-      <c r="Q183" t="n">
+      <c r="U183" t="n">
         <v>8</v>
       </c>
-      <c r="R183" t="n">
+      <c r="V183" t="n">
         <v>6</v>
       </c>
-      <c r="S183" t="n">
+      <c r="W183" t="n">
         <v>4</v>
       </c>
       <c r="Z183" t="n">
         <v>36</v>
       </c>
       <c r="AA183" t="n">
-        <v>4300.56</v>
+        <v>3597.12</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>106004</v>
+        <v>106020</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -12888,21 +12882,21 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>62522833</v>
+        <v>212925785</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>SLB034</t>
+          <t>SSU119</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>SLB034PT</t>
+          <t>SSU119TN</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>SLB034PT</t>
+          <t>SSU119TN</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -12921,15 +12915,15 @@
         </is>
       </c>
       <c r="J184" t="n">
-        <v>599.9</v>
+        <v>299.9</v>
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="L184" t="n">
-        <v>200.54</v>
+        <v>99.92</v>
       </c>
       <c r="M184" t="n">
         <v>1</v>
@@ -12959,12 +12953,12 @@
         <v>18</v>
       </c>
       <c r="AA184" t="n">
-        <v>3609.72</v>
+        <v>1798.56</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>106004</v>
+        <v>106016</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -12972,83 +12966,62 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>164567877</v>
+        <v>226773781</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>SLB034</t>
-        </is>
-      </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>SLB034TN</t>
-        </is>
-      </c>
-      <c r="F185" t="inlineStr">
-        <is>
-          <t>SLB034TN</t>
-        </is>
-      </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>MASCULINO</t>
-        </is>
-      </c>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>TENIS</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>INVERNO</t>
-        </is>
-      </c>
-      <c r="J185" t="n">
-        <v>599.9</v>
-      </c>
-      <c r="K185" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
+          <t>PAB078</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>PAB078CF</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>PAB078CF</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="n"/>
+      <c r="H185" s="2" t="n"/>
+      <c r="I185" s="2" t="n"/>
+      <c r="J185" s="2" t="n"/>
+      <c r="K185" s="2" t="n"/>
       <c r="L185" t="n">
-        <v>200.54</v>
+        <v>149.31</v>
       </c>
       <c r="M185" t="n">
         <v>1</v>
       </c>
+      <c r="N185" t="n">
+        <v>1</v>
+      </c>
+      <c r="O185" t="n">
+        <v>3</v>
+      </c>
+      <c r="P185" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q185" t="n">
+        <v>4</v>
+      </c>
       <c r="R185" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S185" t="n">
-        <v>3</v>
-      </c>
-      <c r="T185" t="n">
-        <v>4</v>
-      </c>
-      <c r="U185" t="n">
-        <v>4</v>
-      </c>
-      <c r="V185" t="n">
-        <v>3</v>
-      </c>
-      <c r="W185" t="n">
-        <v>2</v>
-      </c>
-      <c r="X185" t="n">
         <v>1</v>
       </c>
       <c r="Z185" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AA185" t="n">
-        <v>3609.72</v>
+        <v>2239.65</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>106004</v>
+        <v>106016</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -13056,83 +13029,62 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>209207783</v>
+        <v>227869440</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>SVZ500</t>
-        </is>
-      </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>SVZ500CF</t>
-        </is>
-      </c>
-      <c r="F186" t="inlineStr">
-        <is>
-          <t>SVZ500CF</t>
-        </is>
-      </c>
-      <c r="G186" t="inlineStr">
-        <is>
-          <t>MASCULINO</t>
-        </is>
-      </c>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>TENIS</t>
-        </is>
-      </c>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>CLASSICO</t>
-        </is>
-      </c>
-      <c r="J186" t="n">
-        <v>539.9</v>
-      </c>
-      <c r="K186" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
+          <t>PAB078</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>PAB078VO</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>PAB078VO</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="n"/>
+      <c r="H186" s="2" t="n"/>
+      <c r="I186" s="2" t="n"/>
+      <c r="J186" s="2" t="n"/>
+      <c r="K186" s="2" t="n"/>
       <c r="L186" t="n">
-        <v>174.65</v>
+        <v>149.31</v>
       </c>
       <c r="M186" t="n">
         <v>1</v>
       </c>
+      <c r="N186" t="n">
+        <v>1</v>
+      </c>
+      <c r="O186" t="n">
+        <v>2</v>
+      </c>
+      <c r="P186" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q186" t="n">
+        <v>3</v>
+      </c>
       <c r="R186" t="n">
         <v>2</v>
       </c>
       <c r="S186" t="n">
-        <v>4</v>
-      </c>
-      <c r="T186" t="n">
-        <v>5</v>
-      </c>
-      <c r="U186" t="n">
-        <v>5</v>
-      </c>
-      <c r="V186" t="n">
-        <v>4</v>
-      </c>
-      <c r="W186" t="n">
-        <v>3</v>
-      </c>
-      <c r="X186" t="n">
         <v>1</v>
       </c>
       <c r="Z186" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="AA186" t="n">
-        <v>4191.6</v>
+        <v>1791.72</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>106004</v>
+        <v>106016</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -13140,21 +13092,21 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>226799440</v>
+        <v>226799259</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>WSCR54</t>
+          <t>WCL202</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
         <is>
-          <t>WSCR54BC</t>
+          <t>WCL202CA</t>
         </is>
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>WSCR54BC</t>
+          <t>WCL202CA</t>
         </is>
       </c>
       <c r="G187" s="2" t="n"/>
@@ -13163,7 +13115,7 @@
       <c r="J187" s="2" t="n"/>
       <c r="K187" s="2" t="n"/>
       <c r="L187" t="n">
-        <v>211.68</v>
+        <v>124.7</v>
       </c>
       <c r="M187" t="n">
         <v>1</v>
@@ -13172,13 +13124,13 @@
         <v>1</v>
       </c>
       <c r="O187" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P187" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q187" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R187" t="n">
         <v>2</v>
@@ -13187,15 +13139,15 @@
         <v>1</v>
       </c>
       <c r="Z187" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AA187" t="n">
-        <v>3175.2</v>
+        <v>1496.4</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>106004</v>
+        <v>106016</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -13203,21 +13155,21 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>226799445</v>
+        <v>226799260</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>WSCR57</t>
+          <t>WCL203</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>WSCR57BI</t>
+          <t>WCL203CF</t>
         </is>
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>WSCR57BI</t>
+          <t>WCL203CF</t>
         </is>
       </c>
       <c r="G188" s="2" t="n"/>
@@ -13226,7 +13178,7 @@
       <c r="J188" s="2" t="n"/>
       <c r="K188" s="2" t="n"/>
       <c r="L188" t="n">
-        <v>159.25</v>
+        <v>145.33</v>
       </c>
       <c r="M188" t="n">
         <v>1</v>
@@ -13253,12 +13205,12 @@
         <v>18</v>
       </c>
       <c r="AA188" t="n">
-        <v>2866.5</v>
+        <v>2615.94</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>106004</v>
+        <v>106016</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -13266,21 +13218,21 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>226799459</v>
+        <v>226799261</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>WSCR89</t>
+          <t>WCL204</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>WSCR89TN</t>
+          <t>WCL204CA</t>
         </is>
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>WSCR89TN</t>
+          <t>WCL204CA</t>
         </is>
       </c>
       <c r="G189" s="2" t="n"/>
@@ -13289,7 +13241,7 @@
       <c r="J189" s="2" t="n"/>
       <c r="K189" s="2" t="n"/>
       <c r="L189" t="n">
-        <v>161.58</v>
+        <v>154.12</v>
       </c>
       <c r="M189" t="n">
         <v>1</v>
@@ -13316,12 +13268,12 @@
         <v>18</v>
       </c>
       <c r="AA189" t="n">
-        <v>2908.44</v>
+        <v>2774.16</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>106006</v>
+        <v>106004</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -13329,56 +13281,83 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>226772776</v>
+        <v>99069512</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>ASF182</t>
-        </is>
-      </c>
-      <c r="E190" s="2" t="inlineStr">
-        <is>
-          <t>ASF182MM</t>
-        </is>
-      </c>
-      <c r="F190" s="2" t="inlineStr">
-        <is>
-          <t>ASF182MM</t>
-        </is>
-      </c>
-      <c r="G190" s="2" t="n"/>
-      <c r="H190" s="2" t="n"/>
-      <c r="I190" s="2" t="n"/>
-      <c r="J190" s="2" t="n"/>
-      <c r="K190" s="2" t="n"/>
+          <t>ADP160</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>ADP160CF</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>ADP160CF</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>MOCASSIM</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J190" t="n">
+        <v>439.9</v>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="L190" t="n">
-        <v>64.34999999999999</v>
+        <v>148.03</v>
       </c>
       <c r="M190" t="n">
         <v>1</v>
       </c>
-      <c r="Q190" t="n">
-        <v>4</v>
+      <c r="R190" t="n">
+        <v>2</v>
       </c>
       <c r="S190" t="n">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="T190" t="n">
+        <v>5</v>
       </c>
       <c r="U190" t="n">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="V190" t="n">
+        <v>4</v>
       </c>
       <c r="W190" t="n">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="X190" t="n">
+        <v>1</v>
       </c>
       <c r="Z190" t="n">
         <v>24</v>
       </c>
       <c r="AA190" t="n">
-        <v>1544.4</v>
+        <v>3552.72</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>106006</v>
+        <v>106004</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -13386,21 +13365,21 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1213706</v>
+        <v>56456539</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>ASF182</t>
+          <t>ASF950</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>ASF182PT</t>
+          <t>ASF950TP</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>ASF182PT</t>
+          <t>ASF950TP</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -13415,11 +13394,11 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>CLASSICO</t>
+          <t>VERAO</t>
         </is>
       </c>
       <c r="J191" t="n">
-        <v>199.9</v>
+        <v>399.9</v>
       </c>
       <c r="K191" t="inlineStr">
         <is>
@@ -13427,33 +13406,42 @@
         </is>
       </c>
       <c r="L191" t="n">
-        <v>64.34999999999999</v>
+        <v>124.86</v>
       </c>
       <c r="M191" t="n">
         <v>1</v>
       </c>
-      <c r="Q191" t="n">
-        <v>4</v>
+      <c r="R191" t="n">
+        <v>2</v>
       </c>
       <c r="S191" t="n">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="T191" t="n">
+        <v>5</v>
       </c>
       <c r="U191" t="n">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="V191" t="n">
+        <v>4</v>
       </c>
       <c r="W191" t="n">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="X191" t="n">
+        <v>1</v>
       </c>
       <c r="Z191" t="n">
         <v>24</v>
       </c>
       <c r="AA191" t="n">
-        <v>1544.4</v>
+        <v>2996.64</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>106017</v>
+        <v>106004</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -13461,21 +13449,21 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>156352241</v>
+        <v>63032743</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>PABR56</t>
+          <t>PRAD44</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>PABR56CM</t>
+          <t>PRAD44TP</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>PABR56CM</t>
+          <t>PRAD44TP</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -13485,7 +13473,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>ANABELA</t>
+          <t>SANDALIA BIRKEN</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -13502,7 +13490,7 @@
         </is>
       </c>
       <c r="L192" t="n">
-        <v>121.28</v>
+        <v>119.46</v>
       </c>
       <c r="M192" t="n">
         <v>1</v>
@@ -13511,30 +13499,30 @@
         <v>2</v>
       </c>
       <c r="O192" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P192" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="Q192" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="R192" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S192" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Z192" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="AA192" t="n">
-        <v>2183.04</v>
+        <v>4300.56</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>106017</v>
+        <v>106004</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -13542,31 +13530,31 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>156352242</v>
+        <v>62522833</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>PABR56</t>
+          <t>SLB034</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>PABR56MH</t>
+          <t>SLB034PT</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>PABR56MH</t>
+          <t>SLB034PT</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>FEMININO</t>
+          <t>MASCULINO</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>ANABELA</t>
+          <t>TENIS</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -13575,7 +13563,7 @@
         </is>
       </c>
       <c r="J193" t="n">
-        <v>299.9</v>
+        <v>599.9</v>
       </c>
       <c r="K193" t="inlineStr">
         <is>
@@ -13583,39 +13571,42 @@
         </is>
       </c>
       <c r="L193" t="n">
-        <v>121.28</v>
+        <v>200.54</v>
       </c>
       <c r="M193" t="n">
         <v>1</v>
       </c>
-      <c r="N193" t="n">
-        <v>2</v>
-      </c>
-      <c r="O193" t="n">
-        <v>3</v>
-      </c>
-      <c r="P193" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q193" t="n">
-        <v>4</v>
-      </c>
       <c r="R193" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S193" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="T193" t="n">
+        <v>4</v>
+      </c>
+      <c r="U193" t="n">
+        <v>4</v>
+      </c>
+      <c r="V193" t="n">
+        <v>3</v>
+      </c>
+      <c r="W193" t="n">
+        <v>2</v>
+      </c>
+      <c r="X193" t="n">
+        <v>1</v>
       </c>
       <c r="Z193" t="n">
         <v>18</v>
       </c>
       <c r="AA193" t="n">
-        <v>2183.04</v>
+        <v>3609.72</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>106017</v>
+        <v>106004</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -13623,56 +13614,707 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>226773817</v>
+        <v>164567877</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>PABR80</t>
-        </is>
-      </c>
-      <c r="E194" s="2" t="inlineStr">
-        <is>
-          <t>PABR80FD</t>
-        </is>
-      </c>
-      <c r="F194" s="2" t="inlineStr">
-        <is>
-          <t>PABR80FD</t>
-        </is>
-      </c>
-      <c r="G194" s="2" t="n"/>
-      <c r="H194" s="2" t="n"/>
-      <c r="I194" s="2" t="n"/>
-      <c r="J194" s="2" t="n"/>
-      <c r="K194" s="2" t="n"/>
+          <t>SLB034</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>SLB034TN</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>SLB034TN</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J194" t="n">
+        <v>599.9</v>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
       <c r="L194" t="n">
-        <v>142.1</v>
+        <v>200.54</v>
       </c>
       <c r="M194" t="n">
         <v>1</v>
       </c>
-      <c r="N194" t="n">
-        <v>2</v>
-      </c>
-      <c r="O194" t="n">
-        <v>3</v>
-      </c>
-      <c r="P194" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q194" t="n">
-        <v>4</v>
-      </c>
       <c r="R194" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S194" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="T194" t="n">
+        <v>4</v>
+      </c>
+      <c r="U194" t="n">
+        <v>4</v>
+      </c>
+      <c r="V194" t="n">
+        <v>3</v>
+      </c>
+      <c r="W194" t="n">
+        <v>2</v>
+      </c>
+      <c r="X194" t="n">
+        <v>1</v>
       </c>
       <c r="Z194" t="n">
         <v>18</v>
       </c>
       <c r="AA194" t="n">
+        <v>3609.72</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>106004</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>FQ - BARRA SH. 1</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>209207783</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>SVZ500</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>SVZ500CF</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>SVZ500CF</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J195" t="n">
+        <v>539.9</v>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L195" t="n">
+        <v>174.65</v>
+      </c>
+      <c r="M195" t="n">
+        <v>1</v>
+      </c>
+      <c r="R195" t="n">
+        <v>2</v>
+      </c>
+      <c r="S195" t="n">
+        <v>4</v>
+      </c>
+      <c r="T195" t="n">
+        <v>5</v>
+      </c>
+      <c r="U195" t="n">
+        <v>5</v>
+      </c>
+      <c r="V195" t="n">
+        <v>4</v>
+      </c>
+      <c r="W195" t="n">
+        <v>3</v>
+      </c>
+      <c r="X195" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z195" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA195" t="n">
+        <v>4191.6</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>106004</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>FQ - BARRA SH. 1</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>226799440</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>WSCR54</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>WSCR54BC</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>WSCR54BC</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="n"/>
+      <c r="H196" s="2" t="n"/>
+      <c r="I196" s="2" t="n"/>
+      <c r="J196" s="2" t="n"/>
+      <c r="K196" s="2" t="n"/>
+      <c r="L196" t="n">
+        <v>211.68</v>
+      </c>
+      <c r="M196" t="n">
+        <v>1</v>
+      </c>
+      <c r="N196" t="n">
+        <v>1</v>
+      </c>
+      <c r="O196" t="n">
+        <v>3</v>
+      </c>
+      <c r="P196" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>4</v>
+      </c>
+      <c r="R196" t="n">
+        <v>2</v>
+      </c>
+      <c r="S196" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z196" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA196" t="n">
+        <v>3175.2</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>106004</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>FQ - BARRA SH. 1</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>226799445</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>WSCR57</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
+          <t>WSCR57BI</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t>WSCR57BI</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="n"/>
+      <c r="H197" s="2" t="n"/>
+      <c r="I197" s="2" t="n"/>
+      <c r="J197" s="2" t="n"/>
+      <c r="K197" s="2" t="n"/>
+      <c r="L197" t="n">
+        <v>159.25</v>
+      </c>
+      <c r="M197" t="n">
+        <v>1</v>
+      </c>
+      <c r="N197" t="n">
+        <v>2</v>
+      </c>
+      <c r="O197" t="n">
+        <v>3</v>
+      </c>
+      <c r="P197" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q197" t="n">
+        <v>4</v>
+      </c>
+      <c r="R197" t="n">
+        <v>3</v>
+      </c>
+      <c r="S197" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z197" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA197" t="n">
+        <v>2866.5</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>106004</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>FQ - BARRA SH. 1</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>226799459</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>WSCR89</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>WSCR89TN</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>WSCR89TN</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="n"/>
+      <c r="H198" s="2" t="n"/>
+      <c r="I198" s="2" t="n"/>
+      <c r="J198" s="2" t="n"/>
+      <c r="K198" s="2" t="n"/>
+      <c r="L198" t="n">
+        <v>161.58</v>
+      </c>
+      <c r="M198" t="n">
+        <v>1</v>
+      </c>
+      <c r="N198" t="n">
+        <v>2</v>
+      </c>
+      <c r="O198" t="n">
+        <v>3</v>
+      </c>
+      <c r="P198" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q198" t="n">
+        <v>4</v>
+      </c>
+      <c r="R198" t="n">
+        <v>3</v>
+      </c>
+      <c r="S198" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z198" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA198" t="n">
+        <v>2908.44</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>106006</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>FQ - BARRA SH. 1</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>226772776</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>ASF182</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>ASF182MM</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>ASF182MM</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="n"/>
+      <c r="H199" s="2" t="n"/>
+      <c r="I199" s="2" t="n"/>
+      <c r="J199" s="2" t="n"/>
+      <c r="K199" s="2" t="n"/>
+      <c r="L199" t="n">
+        <v>64.34999999999999</v>
+      </c>
+      <c r="M199" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q199" t="n">
+        <v>4</v>
+      </c>
+      <c r="S199" t="n">
+        <v>8</v>
+      </c>
+      <c r="U199" t="n">
+        <v>8</v>
+      </c>
+      <c r="W199" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z199" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA199" t="n">
+        <v>1544.4</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>106006</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>FQ - BARRA SH. 1</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>1213706</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>ASF182</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>ASF182PT</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>ASF182PT</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>SANDALIA</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J200" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L200" t="n">
+        <v>64.34999999999999</v>
+      </c>
+      <c r="M200" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q200" t="n">
+        <v>4</v>
+      </c>
+      <c r="S200" t="n">
+        <v>8</v>
+      </c>
+      <c r="U200" t="n">
+        <v>8</v>
+      </c>
+      <c r="W200" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z200" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA200" t="n">
+        <v>1544.4</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>106017</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>FQ - BARRA SH. 1</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>156352241</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>PABR56</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>PABR56CM</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>PABR56CM</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>ANABELA</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J201" t="n">
+        <v>299.9</v>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L201" t="n">
+        <v>121.28</v>
+      </c>
+      <c r="M201" t="n">
+        <v>1</v>
+      </c>
+      <c r="N201" t="n">
+        <v>2</v>
+      </c>
+      <c r="O201" t="n">
+        <v>3</v>
+      </c>
+      <c r="P201" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q201" t="n">
+        <v>4</v>
+      </c>
+      <c r="R201" t="n">
+        <v>3</v>
+      </c>
+      <c r="S201" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z201" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA201" t="n">
+        <v>2183.04</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>106017</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>FQ - BARRA SH. 1</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>156352242</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>PABR56</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>PABR56MH</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>PABR56MH</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>ANABELA</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J202" t="n">
+        <v>299.9</v>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L202" t="n">
+        <v>121.28</v>
+      </c>
+      <c r="M202" t="n">
+        <v>1</v>
+      </c>
+      <c r="N202" t="n">
+        <v>2</v>
+      </c>
+      <c r="O202" t="n">
+        <v>3</v>
+      </c>
+      <c r="P202" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q202" t="n">
+        <v>4</v>
+      </c>
+      <c r="R202" t="n">
+        <v>3</v>
+      </c>
+      <c r="S202" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z202" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA202" t="n">
+        <v>2183.04</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>106017</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>FQ - BARRA SH. 1</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>226773817</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>PABR80</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>PABR80FD</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>PABR80FD</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="n"/>
+      <c r="H203" s="2" t="n"/>
+      <c r="I203" s="2" t="n"/>
+      <c r="J203" s="2" t="n"/>
+      <c r="K203" s="2" t="n"/>
+      <c r="L203" t="n">
+        <v>142.1</v>
+      </c>
+      <c r="M203" t="n">
+        <v>1</v>
+      </c>
+      <c r="N203" t="n">
+        <v>2</v>
+      </c>
+      <c r="O203" t="n">
+        <v>3</v>
+      </c>
+      <c r="P203" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q203" t="n">
+        <v>4</v>
+      </c>
+      <c r="R203" t="n">
+        <v>3</v>
+      </c>
+      <c r="S203" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z203" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA203" t="n">
         <v>2557.8</v>
       </c>
     </row>
@@ -14195,15 +14837,26 @@
           <t>CALCADOS KARYBY LTDA</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>B2_RelB2bCarrinhoExcel-18h58.xlsx</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEM ARQUIVO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>75</v>
       </c>
+      <c r="G14" t="n">
+        <v>75</v>
+      </c>
       <c r="H14" t="n">
+        <v>10917.87</v>
+      </c>
+      <c r="I14" t="n">
         <v>10917.87</v>
       </c>
     </row>
@@ -14332,15 +14985,26 @@
           <t>ZOTTO CALCADOS LTDA</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>B1_2_RelB2bCarrinhoExcel-18h58.xlsx</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEM ARQUIVO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>114</v>
       </c>
+      <c r="G18" t="n">
+        <v>114</v>
+      </c>
       <c r="H18" t="n">
+        <v>11390.88</v>
+      </c>
+      <c r="I18" t="n">
         <v>11390.88</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Eldorado order 105722
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9PfgDEdKqrS7U5PG39u7r
</commit_message>
<xml_diff>
--- a/pedidos/Pedidos_Fev27_Unificado.xlsx
+++ b/pedidos/Pedidos_Fev27_Unificado.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA274"/>
+  <dimension ref="A1:AA280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19041,6 +19041,474 @@
       </c>
       <c r="AA274" t="n">
         <v>1095.84</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>105722</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>SH. ELDORADO</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>134703902</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>WSC330</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>WSC330BC</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>WSC330BC</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J275" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L275" t="n">
+        <v>76.86</v>
+      </c>
+      <c r="M275" t="n">
+        <v>1</v>
+      </c>
+      <c r="N275" t="n">
+        <v>1</v>
+      </c>
+      <c r="O275" t="n">
+        <v>3</v>
+      </c>
+      <c r="P275" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q275" t="n">
+        <v>4</v>
+      </c>
+      <c r="R275" t="n">
+        <v>3</v>
+      </c>
+      <c r="S275" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z275" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA275" t="n">
+        <v>1383.48</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>105722</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>SH. ELDORADO</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>226799278</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>WSC330</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>WSC330OU</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>WSC330OU</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="n"/>
+      <c r="H276" s="2" t="n"/>
+      <c r="I276" s="2" t="n"/>
+      <c r="J276" s="2" t="n"/>
+      <c r="K276" s="2" t="n"/>
+      <c r="L276" t="n">
+        <v>68.31999999999999</v>
+      </c>
+      <c r="M276" t="n">
+        <v>1</v>
+      </c>
+      <c r="N276" t="n">
+        <v>2</v>
+      </c>
+      <c r="O276" t="n">
+        <v>4</v>
+      </c>
+      <c r="P276" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q276" t="n">
+        <v>6</v>
+      </c>
+      <c r="R276" t="n">
+        <v>4</v>
+      </c>
+      <c r="S276" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z276" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA276" t="n">
+        <v>1639.68</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>105722</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>SH. ELDORADO</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>147983439</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>WSC432</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>WSC432AW</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>WSC432AW</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J277" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L277" t="n">
+        <v>68.31999999999999</v>
+      </c>
+      <c r="M277" t="n">
+        <v>1</v>
+      </c>
+      <c r="N277" t="n">
+        <v>1</v>
+      </c>
+      <c r="O277" t="n">
+        <v>3</v>
+      </c>
+      <c r="P277" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q277" t="n">
+        <v>4</v>
+      </c>
+      <c r="R277" t="n">
+        <v>3</v>
+      </c>
+      <c r="S277" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z277" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA277" t="n">
+        <v>1229.76</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>105722</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>SH. ELDORADO</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>137619676</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>WSCR61</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>WSCR61AR</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>WSCR61AR</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J278" t="n">
+        <v>399.9</v>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L278" t="n">
+        <v>118.83</v>
+      </c>
+      <c r="M278" t="n">
+        <v>1</v>
+      </c>
+      <c r="N278" t="n">
+        <v>1</v>
+      </c>
+      <c r="O278" t="n">
+        <v>3</v>
+      </c>
+      <c r="P278" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q278" t="n">
+        <v>4</v>
+      </c>
+      <c r="R278" t="n">
+        <v>3</v>
+      </c>
+      <c r="S278" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z278" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA278" t="n">
+        <v>2138.94</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>105722</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>SH. ELDORADO</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>170929723</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>WSCR61</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>WSCR61FD</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>WSCR61FD</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J279" t="n">
+        <v>399.9</v>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L279" t="n">
+        <v>118.83</v>
+      </c>
+      <c r="M279" t="n">
+        <v>1</v>
+      </c>
+      <c r="N279" t="n">
+        <v>1</v>
+      </c>
+      <c r="O279" t="n">
+        <v>3</v>
+      </c>
+      <c r="P279" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q279" t="n">
+        <v>4</v>
+      </c>
+      <c r="R279" t="n">
+        <v>3</v>
+      </c>
+      <c r="S279" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z279" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA279" t="n">
+        <v>2138.94</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>105722</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>SH. ELDORADO</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>137619678</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>WSCR61</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>WSCR61PT</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>WSCR61PT</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J280" t="n">
+        <v>399.9</v>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L280" t="n">
+        <v>118.83</v>
+      </c>
+      <c r="M280" t="n">
+        <v>1</v>
+      </c>
+      <c r="N280" t="n">
+        <v>1</v>
+      </c>
+      <c r="O280" t="n">
+        <v>3</v>
+      </c>
+      <c r="P280" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q280" t="n">
+        <v>4</v>
+      </c>
+      <c r="R280" t="n">
+        <v>3</v>
+      </c>
+      <c r="S280" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z280" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA280" t="n">
+        <v>2138.94</v>
       </c>
     </row>
   </sheetData>
@@ -20524,15 +20992,26 @@
           <t>MASSEY CALCADOS LTDA</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>5876a4d7-RelB2bCarrinhoExcel-19h04.xlsx</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEM ARQUIVO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F40" t="n">
         <v>114</v>
       </c>
+      <c r="G40" t="n">
+        <v>114</v>
+      </c>
       <c r="H40" t="n">
+        <v>10669.74</v>
+      </c>
+      <c r="I40" t="n">
         <v>10669.74</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SH Park Sul orders
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9PfgDEdKqrS7U5PG39u7r
</commit_message>
<xml_diff>
--- a/pedidos/Pedidos_Fev27_Unificado.xlsx
+++ b/pedidos/Pedidos_Fev27_Unificado.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA280"/>
+  <dimension ref="A1:AA294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19509,6 +19509,909 @@
       </c>
       <c r="AA280" t="n">
         <v>2138.94</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>105839</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>12078368</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>HMO032</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>HMO032CF</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>HMO032CF</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>BOLSA MASCULINA</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J281" t="n">
+        <v>999.9</v>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L281" t="n">
+        <v>348</v>
+      </c>
+      <c r="M281" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y281" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z281" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA281" t="n">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>105839</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>12078369</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>HMO032</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>HMO032PT</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>HMO032PT</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>BOLSA MASCULINA</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J282" t="n">
+        <v>999.9</v>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L282" t="n">
+        <v>348</v>
+      </c>
+      <c r="M282" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y282" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z282" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA282" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>105840</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>13224</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>HMO101</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>HMO101CF</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>HMO101CF</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>BOLSA MASCULINA</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J283" t="n">
+        <v>899.9</v>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L283" t="n">
+        <v>254.27</v>
+      </c>
+      <c r="M283" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y283" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z283" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA283" t="n">
+        <v>254.27</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>105841</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>227869440</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>PAB078</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>PAB078VO</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>PAB078VO</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="n"/>
+      <c r="H284" s="2" t="n"/>
+      <c r="I284" s="2" t="n"/>
+      <c r="J284" s="2" t="n"/>
+      <c r="K284" s="2" t="n"/>
+      <c r="L284" t="n">
+        <v>149.31</v>
+      </c>
+      <c r="M284" t="n">
+        <v>1</v>
+      </c>
+      <c r="N284" t="n">
+        <v>1</v>
+      </c>
+      <c r="O284" t="n">
+        <v>2</v>
+      </c>
+      <c r="P284" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q284" t="n">
+        <v>2</v>
+      </c>
+      <c r="R284" t="n">
+        <v>1</v>
+      </c>
+      <c r="S284" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z284" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA284" t="n">
+        <v>1343.79</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>105841</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>164260186</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>WCL099</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>WCL099CF</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>WCL099CF</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>MOCASSIM</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J285" t="n">
+        <v>269.9</v>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L285" t="n">
+        <v>89.06999999999999</v>
+      </c>
+      <c r="M285" t="n">
+        <v>1</v>
+      </c>
+      <c r="N285" t="n">
+        <v>1</v>
+      </c>
+      <c r="O285" t="n">
+        <v>2</v>
+      </c>
+      <c r="P285" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q285" t="n">
+        <v>2</v>
+      </c>
+      <c r="R285" t="n">
+        <v>1</v>
+      </c>
+      <c r="S285" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z285" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA285" t="n">
+        <v>801.63</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>105841</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>226799259</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>WCL202</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>WCL202CA</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>WCL202CA</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="n"/>
+      <c r="H286" s="2" t="n"/>
+      <c r="I286" s="2" t="n"/>
+      <c r="J286" s="2" t="n"/>
+      <c r="K286" s="2" t="n"/>
+      <c r="L286" t="n">
+        <v>124.7</v>
+      </c>
+      <c r="M286" t="n">
+        <v>1</v>
+      </c>
+      <c r="N286" t="n">
+        <v>1</v>
+      </c>
+      <c r="O286" t="n">
+        <v>2</v>
+      </c>
+      <c r="P286" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q286" t="n">
+        <v>2</v>
+      </c>
+      <c r="R286" t="n">
+        <v>1</v>
+      </c>
+      <c r="S286" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z286" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA286" t="n">
+        <v>1122.3</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>105842</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>226773985</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>PMD407</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>PMD407CF</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>PMD407CF</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="n"/>
+      <c r="H287" s="2" t="n"/>
+      <c r="I287" s="2" t="n"/>
+      <c r="J287" s="2" t="n"/>
+      <c r="K287" s="2" t="n"/>
+      <c r="L287" t="n">
+        <v>110.18</v>
+      </c>
+      <c r="M287" t="n">
+        <v>1</v>
+      </c>
+      <c r="N287" t="n">
+        <v>1</v>
+      </c>
+      <c r="O287" t="n">
+        <v>2</v>
+      </c>
+      <c r="P287" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q287" t="n">
+        <v>2</v>
+      </c>
+      <c r="R287" t="n">
+        <v>1</v>
+      </c>
+      <c r="S287" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z287" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA287" t="n">
+        <v>991.62</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>105842</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>226774180</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>PRA732</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>PRA732CF</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>PRA732CF</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="n"/>
+      <c r="H288" s="2" t="n"/>
+      <c r="I288" s="2" t="n"/>
+      <c r="J288" s="2" t="n"/>
+      <c r="K288" s="2" t="n"/>
+      <c r="L288" t="n">
+        <v>61.35</v>
+      </c>
+      <c r="M288" t="n">
+        <v>1</v>
+      </c>
+      <c r="N288" t="n">
+        <v>1</v>
+      </c>
+      <c r="O288" t="n">
+        <v>2</v>
+      </c>
+      <c r="P288" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q288" t="n">
+        <v>2</v>
+      </c>
+      <c r="R288" t="n">
+        <v>1</v>
+      </c>
+      <c r="S288" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z288" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA288" t="n">
+        <v>552.15</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>105842</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>226774181</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>PRA732</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>PRA732VO</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>PRA732VO</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="n"/>
+      <c r="H289" s="2" t="n"/>
+      <c r="I289" s="2" t="n"/>
+      <c r="J289" s="2" t="n"/>
+      <c r="K289" s="2" t="n"/>
+      <c r="L289" t="n">
+        <v>61.35</v>
+      </c>
+      <c r="M289" t="n">
+        <v>1</v>
+      </c>
+      <c r="N289" t="n">
+        <v>1</v>
+      </c>
+      <c r="O289" t="n">
+        <v>2</v>
+      </c>
+      <c r="P289" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q289" t="n">
+        <v>2</v>
+      </c>
+      <c r="R289" t="n">
+        <v>1</v>
+      </c>
+      <c r="S289" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z289" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA289" t="n">
+        <v>552.15</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>105838</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>161296295</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>GBF325</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>GBF325CF</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>GBF325CF</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J290" t="n">
+        <v>469.9</v>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L290" t="n">
+        <v>169.2</v>
+      </c>
+      <c r="M290" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y290" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z290" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA290" t="n">
+        <v>169.2</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>105838</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>58174815</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>GBF445</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>GBF445PT</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>GBF445PT</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J291" t="n">
+        <v>299.9</v>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L291" t="n">
+        <v>122.67</v>
+      </c>
+      <c r="M291" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y291" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z291" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA291" t="n">
+        <v>122.67</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>105838</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>226773215</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>GBF786</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="inlineStr">
+        <is>
+          <t>GBF786CF</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="inlineStr">
+        <is>
+          <t>GBF786CF</t>
+        </is>
+      </c>
+      <c r="G292" s="2" t="n"/>
+      <c r="H292" s="2" t="n"/>
+      <c r="I292" s="2" t="n"/>
+      <c r="J292" s="2" t="n"/>
+      <c r="K292" s="2" t="n"/>
+      <c r="L292" t="n">
+        <v>200.69</v>
+      </c>
+      <c r="M292" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y292" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z292" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA292" t="n">
+        <v>401.38</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>105838</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>177646295</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>GBF827</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>GBF827PT</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>GBF827PT</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J293" t="n">
+        <v>299.9</v>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L293" t="n">
+        <v>85.78</v>
+      </c>
+      <c r="M293" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y293" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z293" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA293" t="n">
+        <v>171.56</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>105843</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>226780324</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>SLG010</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="inlineStr">
+        <is>
+          <t>SLG010PT</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="inlineStr">
+        <is>
+          <t>SLG010PT</t>
+        </is>
+      </c>
+      <c r="G294" s="2" t="n"/>
+      <c r="H294" s="2" t="n"/>
+      <c r="I294" s="2" t="n"/>
+      <c r="J294" s="2" t="n"/>
+      <c r="K294" s="2" t="n"/>
+      <c r="L294" t="n">
+        <v>242.31</v>
+      </c>
+      <c r="M294" t="n">
+        <v>1</v>
+      </c>
+      <c r="R294" t="n">
+        <v>1</v>
+      </c>
+      <c r="S294" t="n">
+        <v>1</v>
+      </c>
+      <c r="T294" t="n">
+        <v>2</v>
+      </c>
+      <c r="U294" t="n">
+        <v>2</v>
+      </c>
+      <c r="V294" t="n">
+        <v>2</v>
+      </c>
+      <c r="W294" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z294" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA294" t="n">
+        <v>2180.79</v>
       </c>
     </row>
   </sheetData>
@@ -19522,7 +20425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21422,6 +22325,228 @@
         <v>3287.52</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>105838</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CLASSE COURO DISTRIBUIDORA</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>RelB2bCarrinhoExcel-19h07.xlsx</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>6</v>
+      </c>
+      <c r="G52" t="n">
+        <v>6</v>
+      </c>
+      <c r="H52" t="n">
+        <v>864.8099999999999</v>
+      </c>
+      <c r="I52" t="n">
+        <v>864.8099999999999</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>105839</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>RAZZAZ ACESSORIOS E ARTIGOS DE COURO LTDA</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2_RelB2bCarrinhoExcel-19h07.xlsx</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>3</v>
+      </c>
+      <c r="G53" t="n">
+        <v>3</v>
+      </c>
+      <c r="H53" t="n">
+        <v>1044</v>
+      </c>
+      <c r="I53" t="n">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>105840</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>BMCG INDUSTRIA E COMERCIO DE COURO LTDA - EPP</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3_RelB2bCarrinhoExcel-19h07.xlsx</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" t="n">
+        <v>254.27</v>
+      </c>
+      <c r="I54" t="n">
+        <v>254.27</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>105841</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CALCADOS KARYBY LTDA</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>4_RelB2bCarrinhoExcel-19h07.xlsx</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>27</v>
+      </c>
+      <c r="G55" t="n">
+        <v>27</v>
+      </c>
+      <c r="H55" t="n">
+        <v>3267.72</v>
+      </c>
+      <c r="I55" t="n">
+        <v>3267.72</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>105842</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>WW EXPORT LTDA</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>5_RelB2bCarrinhoExcel-19h07.xlsx</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>27</v>
+      </c>
+      <c r="G56" t="n">
+        <v>27</v>
+      </c>
+      <c r="H56" t="n">
+        <v>2095.92</v>
+      </c>
+      <c r="I56" t="n">
+        <v>2095.92</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>105843</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>SH. PARK SUL</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>J. B. SHOES INDUSTRIA E COMERCIO DE CALCADOS LTDA - ME</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>RelB2bCarrinhoExcel-19h08.xlsx</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>9</v>
+      </c>
+      <c r="G57" t="n">
+        <v>9</v>
+      </c>
+      <c r="H57" t="n">
+        <v>2180.79</v>
+      </c>
+      <c r="I57" t="n">
+        <v>2180.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Tijuca orders 105822 and 105832
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9PfgDEdKqrS7U5PG39u7r
</commit_message>
<xml_diff>
--- a/pedidos/Pedidos_Fev27_Unificado.xlsx
+++ b/pedidos/Pedidos_Fev27_Unificado.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA550"/>
+  <dimension ref="A1:AA563"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37391,6 +37391,876 @@
         <v>2311.8</v>
       </c>
     </row>
+    <row r="551">
+      <c r="A551" t="n">
+        <v>105822</v>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C551" t="n">
+        <v>198486332</v>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>CAB302</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>CAB302PT</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>CAB302PT</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>SOCIAL</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>VERAO</t>
+        </is>
+      </c>
+      <c r="J551" t="n">
+        <v>699.9</v>
+      </c>
+      <c r="K551" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L551" t="n">
+        <v>250.92</v>
+      </c>
+      <c r="M551" t="n">
+        <v>1</v>
+      </c>
+      <c r="S551" t="n">
+        <v>1</v>
+      </c>
+      <c r="T551" t="n">
+        <v>2</v>
+      </c>
+      <c r="U551" t="n">
+        <v>2</v>
+      </c>
+      <c r="V551" t="n">
+        <v>2</v>
+      </c>
+      <c r="W551" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z551" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA551" t="n">
+        <v>2258.28</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="n">
+        <v>105822</v>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C552" t="n">
+        <v>226772891</v>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>CAR112</t>
+        </is>
+      </c>
+      <c r="E552" s="2" t="inlineStr">
+        <is>
+          <t>CAR112PT</t>
+        </is>
+      </c>
+      <c r="F552" s="2" t="inlineStr">
+        <is>
+          <t>CAR112PT</t>
+        </is>
+      </c>
+      <c r="G552" s="2" t="n"/>
+      <c r="H552" s="2" t="n"/>
+      <c r="I552" s="2" t="n"/>
+      <c r="J552" s="2" t="n"/>
+      <c r="K552" s="2" t="n"/>
+      <c r="L552" t="n">
+        <v>268.14</v>
+      </c>
+      <c r="M552" t="n">
+        <v>1</v>
+      </c>
+      <c r="R552" t="n">
+        <v>1</v>
+      </c>
+      <c r="S552" t="n">
+        <v>2</v>
+      </c>
+      <c r="T552" t="n">
+        <v>3</v>
+      </c>
+      <c r="U552" t="n">
+        <v>2</v>
+      </c>
+      <c r="V552" t="n">
+        <v>2</v>
+      </c>
+      <c r="W552" t="n">
+        <v>1</v>
+      </c>
+      <c r="X552" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z552" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA552" t="n">
+        <v>3217.68</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="n">
+        <v>105822</v>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C553" t="n">
+        <v>226772892</v>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>CAR113</t>
+        </is>
+      </c>
+      <c r="E553" s="2" t="inlineStr">
+        <is>
+          <t>CAR113CF</t>
+        </is>
+      </c>
+      <c r="F553" s="2" t="inlineStr">
+        <is>
+          <t>CAR113CF</t>
+        </is>
+      </c>
+      <c r="G553" s="2" t="n"/>
+      <c r="H553" s="2" t="n"/>
+      <c r="I553" s="2" t="n"/>
+      <c r="J553" s="2" t="n"/>
+      <c r="K553" s="2" t="n"/>
+      <c r="L553" t="n">
+        <v>268.14</v>
+      </c>
+      <c r="M553" t="n">
+        <v>1</v>
+      </c>
+      <c r="R553" t="n">
+        <v>1</v>
+      </c>
+      <c r="S553" t="n">
+        <v>2</v>
+      </c>
+      <c r="T553" t="n">
+        <v>3</v>
+      </c>
+      <c r="U553" t="n">
+        <v>2</v>
+      </c>
+      <c r="V553" t="n">
+        <v>2</v>
+      </c>
+      <c r="W553" t="n">
+        <v>1</v>
+      </c>
+      <c r="X553" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z553" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA553" t="n">
+        <v>3217.68</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="n">
+        <v>105822</v>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C554" t="n">
+        <v>226772990</v>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>DTR013</t>
+        </is>
+      </c>
+      <c r="E554" s="2" t="inlineStr">
+        <is>
+          <t>DTR013MR</t>
+        </is>
+      </c>
+      <c r="F554" s="2" t="inlineStr">
+        <is>
+          <t>DTR013MR</t>
+        </is>
+      </c>
+      <c r="G554" s="2" t="n"/>
+      <c r="H554" s="2" t="n"/>
+      <c r="I554" s="2" t="n"/>
+      <c r="J554" s="2" t="n"/>
+      <c r="K554" s="2" t="n"/>
+      <c r="L554" t="n">
+        <v>167.28</v>
+      </c>
+      <c r="M554" t="n">
+        <v>1</v>
+      </c>
+      <c r="R554" t="n">
+        <v>1</v>
+      </c>
+      <c r="S554" t="n">
+        <v>2</v>
+      </c>
+      <c r="T554" t="n">
+        <v>3</v>
+      </c>
+      <c r="U554" t="n">
+        <v>4</v>
+      </c>
+      <c r="V554" t="n">
+        <v>3</v>
+      </c>
+      <c r="W554" t="n">
+        <v>1</v>
+      </c>
+      <c r="X554" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z554" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA554" t="n">
+        <v>2509.2</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="n">
+        <v>105822</v>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C555" t="n">
+        <v>226772991</v>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>DTR013</t>
+        </is>
+      </c>
+      <c r="E555" s="2" t="inlineStr">
+        <is>
+          <t>DTR013PT</t>
+        </is>
+      </c>
+      <c r="F555" s="2" t="inlineStr">
+        <is>
+          <t>DTR013PT</t>
+        </is>
+      </c>
+      <c r="G555" s="2" t="n"/>
+      <c r="H555" s="2" t="n"/>
+      <c r="I555" s="2" t="n"/>
+      <c r="J555" s="2" t="n"/>
+      <c r="K555" s="2" t="n"/>
+      <c r="L555" t="n">
+        <v>167.28</v>
+      </c>
+      <c r="M555" t="n">
+        <v>1</v>
+      </c>
+      <c r="R555" t="n">
+        <v>1</v>
+      </c>
+      <c r="S555" t="n">
+        <v>2</v>
+      </c>
+      <c r="T555" t="n">
+        <v>3</v>
+      </c>
+      <c r="U555" t="n">
+        <v>2</v>
+      </c>
+      <c r="V555" t="n">
+        <v>2</v>
+      </c>
+      <c r="W555" t="n">
+        <v>1</v>
+      </c>
+      <c r="X555" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z555" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA555" t="n">
+        <v>2007.36</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="n">
+        <v>105822</v>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C556" t="n">
+        <v>226780323</v>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>SLG010</t>
+        </is>
+      </c>
+      <c r="E556" s="2" t="inlineStr">
+        <is>
+          <t>SLG010MR</t>
+        </is>
+      </c>
+      <c r="F556" s="2" t="inlineStr">
+        <is>
+          <t>SLG010MR</t>
+        </is>
+      </c>
+      <c r="G556" s="2" t="n"/>
+      <c r="H556" s="2" t="n"/>
+      <c r="I556" s="2" t="n"/>
+      <c r="J556" s="2" t="n"/>
+      <c r="K556" s="2" t="n"/>
+      <c r="L556" t="n">
+        <v>242.31</v>
+      </c>
+      <c r="M556" t="n">
+        <v>1</v>
+      </c>
+      <c r="R556" t="n">
+        <v>1</v>
+      </c>
+      <c r="S556" t="n">
+        <v>2</v>
+      </c>
+      <c r="T556" t="n">
+        <v>3</v>
+      </c>
+      <c r="U556" t="n">
+        <v>3</v>
+      </c>
+      <c r="V556" t="n">
+        <v>3</v>
+      </c>
+      <c r="W556" t="n">
+        <v>2</v>
+      </c>
+      <c r="X556" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z556" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA556" t="n">
+        <v>3634.65</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="n">
+        <v>105822</v>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C557" t="n">
+        <v>226780324</v>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>SLG010</t>
+        </is>
+      </c>
+      <c r="E557" s="2" t="inlineStr">
+        <is>
+          <t>SLG010PT</t>
+        </is>
+      </c>
+      <c r="F557" s="2" t="inlineStr">
+        <is>
+          <t>SLG010PT</t>
+        </is>
+      </c>
+      <c r="G557" s="2" t="n"/>
+      <c r="H557" s="2" t="n"/>
+      <c r="I557" s="2" t="n"/>
+      <c r="J557" s="2" t="n"/>
+      <c r="K557" s="2" t="n"/>
+      <c r="L557" t="n">
+        <v>242.31</v>
+      </c>
+      <c r="M557" t="n">
+        <v>1</v>
+      </c>
+      <c r="R557" t="n">
+        <v>1</v>
+      </c>
+      <c r="S557" t="n">
+        <v>2</v>
+      </c>
+      <c r="T557" t="n">
+        <v>3</v>
+      </c>
+      <c r="U557" t="n">
+        <v>3</v>
+      </c>
+      <c r="V557" t="n">
+        <v>3</v>
+      </c>
+      <c r="W557" t="n">
+        <v>2</v>
+      </c>
+      <c r="X557" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z557" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA557" t="n">
+        <v>3634.65</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="n">
+        <v>105832</v>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C558" t="n">
+        <v>226773909</v>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>PAX634</t>
+        </is>
+      </c>
+      <c r="E558" s="2" t="inlineStr">
+        <is>
+          <t>PAX634CA</t>
+        </is>
+      </c>
+      <c r="F558" s="2" t="inlineStr">
+        <is>
+          <t>PAX634CA</t>
+        </is>
+      </c>
+      <c r="G558" s="2" t="n"/>
+      <c r="H558" s="2" t="n"/>
+      <c r="I558" s="2" t="n"/>
+      <c r="J558" s="2" t="n"/>
+      <c r="K558" s="2" t="n"/>
+      <c r="L558" t="n">
+        <v>101.43</v>
+      </c>
+      <c r="M558" t="n">
+        <v>1</v>
+      </c>
+      <c r="N558" t="n">
+        <v>1</v>
+      </c>
+      <c r="O558" t="n">
+        <v>3</v>
+      </c>
+      <c r="P558" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q558" t="n">
+        <v>4</v>
+      </c>
+      <c r="R558" t="n">
+        <v>3</v>
+      </c>
+      <c r="S558" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z558" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA558" t="n">
+        <v>1825.74</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="n">
+        <v>105832</v>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C559" t="n">
+        <v>178969123</v>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>PRA127</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>PRA127CF</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>PRA127CF</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>SANDALIA RASTEIRA</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J559" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="K559" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L559" t="n">
+        <v>61.13</v>
+      </c>
+      <c r="M559" t="n">
+        <v>1</v>
+      </c>
+      <c r="N559" t="n">
+        <v>1</v>
+      </c>
+      <c r="O559" t="n">
+        <v>3</v>
+      </c>
+      <c r="P559" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q559" t="n">
+        <v>4</v>
+      </c>
+      <c r="R559" t="n">
+        <v>3</v>
+      </c>
+      <c r="S559" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z559" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA559" t="n">
+        <v>1100.34</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="n">
+        <v>105832</v>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C560" t="n">
+        <v>226774175</v>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>PRA728</t>
+        </is>
+      </c>
+      <c r="E560" s="2" t="inlineStr">
+        <is>
+          <t>PRA728FD</t>
+        </is>
+      </c>
+      <c r="F560" s="2" t="inlineStr">
+        <is>
+          <t>PRA728FD</t>
+        </is>
+      </c>
+      <c r="G560" s="2" t="n"/>
+      <c r="H560" s="2" t="n"/>
+      <c r="I560" s="2" t="n"/>
+      <c r="J560" s="2" t="n"/>
+      <c r="K560" s="2" t="n"/>
+      <c r="L560" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="M560" t="n">
+        <v>1</v>
+      </c>
+      <c r="N560" t="n">
+        <v>2</v>
+      </c>
+      <c r="O560" t="n">
+        <v>4</v>
+      </c>
+      <c r="P560" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q560" t="n">
+        <v>5</v>
+      </c>
+      <c r="R560" t="n">
+        <v>4</v>
+      </c>
+      <c r="S560" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z560" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA560" t="n">
+        <v>1702.32</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="n">
+        <v>105832</v>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C561" t="n">
+        <v>226774176</v>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>PRA728</t>
+        </is>
+      </c>
+      <c r="E561" s="2" t="inlineStr">
+        <is>
+          <t>PRA728VO</t>
+        </is>
+      </c>
+      <c r="F561" s="2" t="inlineStr">
+        <is>
+          <t>PRA728VO</t>
+        </is>
+      </c>
+      <c r="G561" s="2" t="n"/>
+      <c r="H561" s="2" t="n"/>
+      <c r="I561" s="2" t="n"/>
+      <c r="J561" s="2" t="n"/>
+      <c r="K561" s="2" t="n"/>
+      <c r="L561" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="M561" t="n">
+        <v>1</v>
+      </c>
+      <c r="N561" t="n">
+        <v>1</v>
+      </c>
+      <c r="O561" t="n">
+        <v>3</v>
+      </c>
+      <c r="P561" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q561" t="n">
+        <v>4</v>
+      </c>
+      <c r="R561" t="n">
+        <v>2</v>
+      </c>
+      <c r="S561" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z561" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA561" t="n">
+        <v>1063.95</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="n">
+        <v>105832</v>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C562" t="n">
+        <v>226774179</v>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>PRA730</t>
+        </is>
+      </c>
+      <c r="E562" s="2" t="inlineStr">
+        <is>
+          <t>PRA730CA</t>
+        </is>
+      </c>
+      <c r="F562" s="2" t="inlineStr">
+        <is>
+          <t>PRA730CA</t>
+        </is>
+      </c>
+      <c r="G562" s="2" t="n"/>
+      <c r="H562" s="2" t="n"/>
+      <c r="I562" s="2" t="n"/>
+      <c r="J562" s="2" t="n"/>
+      <c r="K562" s="2" t="n"/>
+      <c r="L562" t="n">
+        <v>108.9</v>
+      </c>
+      <c r="M562" t="n">
+        <v>1</v>
+      </c>
+      <c r="N562" t="n">
+        <v>1</v>
+      </c>
+      <c r="O562" t="n">
+        <v>3</v>
+      </c>
+      <c r="P562" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q562" t="n">
+        <v>3</v>
+      </c>
+      <c r="R562" t="n">
+        <v>3</v>
+      </c>
+      <c r="S562" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z562" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA562" t="n">
+        <v>1633.5</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="n">
+        <v>105832</v>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>SH. TIJUCA</t>
+        </is>
+      </c>
+      <c r="C563" t="n">
+        <v>226799120</v>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>TBC207</t>
+        </is>
+      </c>
+      <c r="E563" s="2" t="inlineStr">
+        <is>
+          <t>TBC207CA</t>
+        </is>
+      </c>
+      <c r="F563" s="2" t="inlineStr">
+        <is>
+          <t>TBC207CA</t>
+        </is>
+      </c>
+      <c r="G563" s="2" t="n"/>
+      <c r="H563" s="2" t="n"/>
+      <c r="I563" s="2" t="n"/>
+      <c r="J563" s="2" t="n"/>
+      <c r="K563" s="2" t="n"/>
+      <c r="L563" t="n">
+        <v>56.96</v>
+      </c>
+      <c r="M563" t="n">
+        <v>1</v>
+      </c>
+      <c r="N563" t="n">
+        <v>2</v>
+      </c>
+      <c r="O563" t="n">
+        <v>4</v>
+      </c>
+      <c r="P563" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q563" t="n">
+        <v>6</v>
+      </c>
+      <c r="R563" t="n">
+        <v>4</v>
+      </c>
+      <c r="S563" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z563" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA563" t="n">
+        <v>1367.04</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -39464,15 +40334,26 @@
           <t>J. B. SHOES INDUSTRIA E COMERCIO DE CALCADOS LTDA - ME</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>1b67292a-RelB2bCarrinhoExcel-19h30.xlsx</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEM ARQUIVO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F56" t="n">
         <v>90</v>
       </c>
+      <c r="G56" t="n">
+        <v>90</v>
+      </c>
       <c r="H56" t="n">
+        <v>20479.5</v>
+      </c>
+      <c r="I56" t="n">
         <v>20479.5</v>
       </c>
     </row>
@@ -39823,15 +40704,26 @@
           <t>FABRICACAO DE CALCADOS PERTHO LTDA</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>7ce5fc48-2_RelB2bCarrinhoExcel-19h30.xlsx</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>SEM ARQUIVO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F66" t="n">
         <v>114</v>
       </c>
+      <c r="G66" t="n">
+        <v>114</v>
+      </c>
       <c r="H66" t="n">
+        <v>8692.889999999999</v>
+      </c>
+      <c r="I66" t="n">
         <v>8692.889999999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Infer departamento/categoria by 6-char reference; default colecao Inverno26
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9PfgDEdKqrS7U5PG39u7r
</commit_message>
<xml_diff>
--- a/pedidos/Pedidos_Fev27_Unificado.xlsx
+++ b/pedidos/Pedidos_Fev27_Unificado.xlsx
@@ -577,7 +577,11 @@
       </c>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" t="n">
@@ -727,7 +731,11 @@
       </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
       <c r="L4" t="n">
@@ -931,7 +939,11 @@
       </c>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
       <c r="L7" t="n">
@@ -994,7 +1006,11 @@
       </c>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
       <c r="L8" t="n">
@@ -1057,7 +1073,11 @@
       </c>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
       <c r="L9" t="n">
@@ -1120,7 +1140,11 @@
       </c>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
       <c r="L10" t="n">
@@ -1183,7 +1207,11 @@
       </c>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" t="n">
@@ -1510,7 +1538,11 @@
       </c>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
       <c r="L16" t="n">
@@ -1573,7 +1605,11 @@
       </c>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
       <c r="L17" t="n">
@@ -1636,7 +1672,11 @@
       </c>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" t="n">
@@ -1687,21 +1727,31 @@
           <t>WSC330</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="n"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L19" t="n">
         <v>68.31999999999999</v>
       </c>
@@ -1924,7 +1974,11 @@
       </c>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
       <c r="L22" t="n">
@@ -1987,7 +2041,11 @@
       </c>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
       <c r="L23" t="n">
@@ -2512,7 +2570,11 @@
       </c>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J31" s="2" t="n"/>
       <c r="K31" s="2" t="n"/>
       <c r="L31" t="n">
@@ -2560,7 +2622,11 @@
       </c>
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
       <c r="L32" t="n">
@@ -2608,7 +2674,11 @@
       </c>
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="2" t="n"/>
       <c r="L33" t="n">
@@ -2788,7 +2858,11 @@
       </c>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
       <c r="L36" t="n">
@@ -2836,7 +2910,11 @@
       </c>
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J37" s="2" t="n"/>
       <c r="K37" s="2" t="n"/>
       <c r="L37" t="n">
@@ -2884,7 +2962,11 @@
       </c>
       <c r="G38" s="2" t="n"/>
       <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="n"/>
       <c r="K38" s="2" t="n"/>
       <c r="L38" t="n">
@@ -3874,7 +3956,11 @@
       </c>
       <c r="G52" s="2" t="n"/>
       <c r="H52" s="2" t="n"/>
-      <c r="I52" s="2" t="n"/>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="n"/>
       <c r="L52" t="n">
@@ -3937,7 +4023,11 @@
       </c>
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="n"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J53" s="2" t="n"/>
       <c r="K53" s="2" t="n"/>
       <c r="L53" t="n">
@@ -3988,21 +4078,39 @@
           <t>SAF126</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="G54" s="2" t="n"/>
-      <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="n"/>
-      <c r="J54" s="2" t="n"/>
-      <c r="K54" s="2" t="n"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>249.9</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="L54" t="n">
         <v>135.3</v>
       </c>
@@ -4150,7 +4258,11 @@
       </c>
       <c r="G56" s="2" t="n"/>
       <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n"/>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J56" s="2" t="n"/>
       <c r="K56" s="2" t="n"/>
       <c r="L56" t="n">
@@ -4720,7 +4832,11 @@
       </c>
       <c r="G64" s="2" t="n"/>
       <c r="H64" s="2" t="n"/>
-      <c r="I64" s="2" t="n"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J64" s="2" t="n"/>
       <c r="K64" s="2" t="n"/>
       <c r="L64" t="n">
@@ -4783,7 +4899,11 @@
       </c>
       <c r="G65" s="2" t="n"/>
       <c r="H65" s="2" t="n"/>
-      <c r="I65" s="2" t="n"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="n"/>
       <c r="L65" t="n">
@@ -4846,7 +4966,11 @@
       </c>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
-      <c r="I66" s="2" t="n"/>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J66" s="2" t="n"/>
       <c r="K66" s="2" t="n"/>
       <c r="L66" t="n">
@@ -5065,21 +5189,39 @@
           <t>SAF126</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="G69" s="2" t="n"/>
-      <c r="H69" s="2" t="n"/>
-      <c r="I69" s="2" t="n"/>
-      <c r="J69" s="2" t="n"/>
-      <c r="K69" s="2" t="n"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>249.9</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="L69" t="n">
         <v>135.3</v>
       </c>
@@ -5815,7 +5957,11 @@
       </c>
       <c r="G78" s="2" t="n"/>
       <c r="H78" s="2" t="n"/>
-      <c r="I78" s="2" t="n"/>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J78" s="2" t="n"/>
       <c r="K78" s="2" t="n"/>
       <c r="L78" t="n">
@@ -6127,7 +6273,11 @@
       </c>
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="2" t="n"/>
-      <c r="I82" s="2" t="n"/>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J82" s="2" t="n"/>
       <c r="K82" s="2" t="n"/>
       <c r="L82" t="n">
@@ -6190,7 +6340,11 @@
       </c>
       <c r="G83" s="2" t="n"/>
       <c r="H83" s="2" t="n"/>
-      <c r="I83" s="2" t="n"/>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J83" s="2" t="n"/>
       <c r="K83" s="2" t="n"/>
       <c r="L83" t="n">
@@ -6253,7 +6407,11 @@
       </c>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n"/>
-      <c r="I84" s="2" t="n"/>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J84" s="2" t="n"/>
       <c r="K84" s="2" t="n"/>
       <c r="L84" t="n">
@@ -6316,7 +6474,11 @@
       </c>
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="2" t="n"/>
-      <c r="I85" s="2" t="n"/>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J85" s="2" t="n"/>
       <c r="K85" s="2" t="n"/>
       <c r="L85" t="n">
@@ -6379,7 +6541,11 @@
       </c>
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="2" t="n"/>
-      <c r="I86" s="2" t="n"/>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J86" s="2" t="n"/>
       <c r="K86" s="2" t="n"/>
       <c r="L86" t="n">
@@ -6442,7 +6608,11 @@
       </c>
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="2" t="n"/>
-      <c r="I87" s="2" t="n"/>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J87" s="2" t="n"/>
       <c r="K87" s="2" t="n"/>
       <c r="L87" t="n">
@@ -6505,7 +6675,11 @@
       </c>
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="2" t="n"/>
-      <c r="I88" s="2" t="n"/>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J88" s="2" t="n"/>
       <c r="K88" s="2" t="n"/>
       <c r="L88" t="n">
@@ -7165,21 +7339,31 @@
           <t>WSC330</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr">
+      <c r="E98" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="F98" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="G98" s="2" t="n"/>
-      <c r="H98" s="2" t="n"/>
-      <c r="I98" s="2" t="n"/>
-      <c r="J98" s="2" t="n"/>
-      <c r="K98" s="2" t="n"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L98" t="n">
         <v>68.31999999999999</v>
       </c>
@@ -7840,7 +8024,11 @@
       </c>
       <c r="G107" s="2" t="n"/>
       <c r="H107" s="2" t="n"/>
-      <c r="I107" s="2" t="n"/>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J107" s="2" t="n"/>
       <c r="K107" s="2" t="n"/>
       <c r="L107" t="n">
@@ -7906,7 +8094,11 @@
       </c>
       <c r="G108" s="2" t="n"/>
       <c r="H108" s="2" t="n"/>
-      <c r="I108" s="2" t="n"/>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J108" s="2" t="n"/>
       <c r="K108" s="2" t="n"/>
       <c r="L108" t="n">
@@ -8557,7 +8749,11 @@
       </c>
       <c r="G116" s="2" t="n"/>
       <c r="H116" s="2" t="n"/>
-      <c r="I116" s="2" t="n"/>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J116" s="2" t="n"/>
       <c r="K116" s="2" t="n"/>
       <c r="L116" t="n">
@@ -8623,7 +8819,11 @@
       </c>
       <c r="G117" s="2" t="n"/>
       <c r="H117" s="2" t="n"/>
-      <c r="I117" s="2" t="n"/>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J117" s="2" t="n"/>
       <c r="K117" s="2" t="n"/>
       <c r="L117" t="n">
@@ -8689,7 +8889,11 @@
       </c>
       <c r="G118" s="2" t="n"/>
       <c r="H118" s="2" t="n"/>
-      <c r="I118" s="2" t="n"/>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J118" s="2" t="n"/>
       <c r="K118" s="2" t="n"/>
       <c r="L118" t="n">
@@ -8755,7 +8959,11 @@
       </c>
       <c r="G119" s="2" t="n"/>
       <c r="H119" s="2" t="n"/>
-      <c r="I119" s="2" t="n"/>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J119" s="2" t="n"/>
       <c r="K119" s="2" t="n"/>
       <c r="L119" t="n">
@@ -9085,7 +9293,11 @@
       </c>
       <c r="G124" s="2" t="n"/>
       <c r="H124" s="2" t="n"/>
-      <c r="I124" s="2" t="n"/>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J124" s="2" t="n"/>
       <c r="K124" s="2" t="n"/>
       <c r="L124" t="n">
@@ -9148,7 +9360,11 @@
       </c>
       <c r="G125" s="2" t="n"/>
       <c r="H125" s="2" t="n"/>
-      <c r="I125" s="2" t="n"/>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J125" s="2" t="n"/>
       <c r="K125" s="2" t="n"/>
       <c r="L125" t="n">
@@ -9211,7 +9427,11 @@
       </c>
       <c r="G126" s="2" t="n"/>
       <c r="H126" s="2" t="n"/>
-      <c r="I126" s="2" t="n"/>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J126" s="2" t="n"/>
       <c r="K126" s="2" t="n"/>
       <c r="L126" t="n">
@@ -10462,7 +10682,11 @@
       </c>
       <c r="G145" s="2" t="n"/>
       <c r="H145" s="2" t="n"/>
-      <c r="I145" s="2" t="n"/>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J145" s="2" t="n"/>
       <c r="K145" s="2" t="n"/>
       <c r="L145" t="n">
@@ -10525,7 +10749,11 @@
       </c>
       <c r="G146" s="2" t="n"/>
       <c r="H146" s="2" t="n"/>
-      <c r="I146" s="2" t="n"/>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J146" s="2" t="n"/>
       <c r="K146" s="2" t="n"/>
       <c r="L146" t="n">
@@ -10588,7 +10816,11 @@
       </c>
       <c r="G147" s="2" t="n"/>
       <c r="H147" s="2" t="n"/>
-      <c r="I147" s="2" t="n"/>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J147" s="2" t="n"/>
       <c r="K147" s="2" t="n"/>
       <c r="L147" t="n">
@@ -10651,7 +10883,11 @@
       </c>
       <c r="G148" s="2" t="n"/>
       <c r="H148" s="2" t="n"/>
-      <c r="I148" s="2" t="n"/>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J148" s="2" t="n"/>
       <c r="K148" s="2" t="n"/>
       <c r="L148" t="n">
@@ -10714,7 +10950,11 @@
       </c>
       <c r="G149" s="2" t="n"/>
       <c r="H149" s="2" t="n"/>
-      <c r="I149" s="2" t="n"/>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J149" s="2" t="n"/>
       <c r="K149" s="2" t="n"/>
       <c r="L149" t="n">
@@ -10777,7 +11017,11 @@
       </c>
       <c r="G150" s="2" t="n"/>
       <c r="H150" s="2" t="n"/>
-      <c r="I150" s="2" t="n"/>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J150" s="2" t="n"/>
       <c r="K150" s="2" t="n"/>
       <c r="L150" t="n">
@@ -10825,7 +11069,11 @@
       </c>
       <c r="G151" s="2" t="n"/>
       <c r="H151" s="2" t="n"/>
-      <c r="I151" s="2" t="n"/>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J151" s="2" t="n"/>
       <c r="K151" s="2" t="n"/>
       <c r="L151" t="n">
@@ -10873,7 +11121,11 @@
       </c>
       <c r="G152" s="2" t="n"/>
       <c r="H152" s="2" t="n"/>
-      <c r="I152" s="2" t="n"/>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J152" s="2" t="n"/>
       <c r="K152" s="2" t="n"/>
       <c r="L152" t="n">
@@ -10921,7 +11173,11 @@
       </c>
       <c r="G153" s="2" t="n"/>
       <c r="H153" s="2" t="n"/>
-      <c r="I153" s="2" t="n"/>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J153" s="2" t="n"/>
       <c r="K153" s="2" t="n"/>
       <c r="L153" t="n">
@@ -10969,7 +11225,11 @@
       </c>
       <c r="G154" s="2" t="n"/>
       <c r="H154" s="2" t="n"/>
-      <c r="I154" s="2" t="n"/>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J154" s="2" t="n"/>
       <c r="K154" s="2" t="n"/>
       <c r="L154" t="n">
@@ -11281,7 +11541,11 @@
       </c>
       <c r="G159" s="2" t="n"/>
       <c r="H159" s="2" t="n"/>
-      <c r="I159" s="2" t="n"/>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J159" s="2" t="n"/>
       <c r="K159" s="2" t="n"/>
       <c r="L159" t="n">
@@ -11329,7 +11593,11 @@
       </c>
       <c r="G160" s="2" t="n"/>
       <c r="H160" s="2" t="n"/>
-      <c r="I160" s="2" t="n"/>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J160" s="2" t="n"/>
       <c r="K160" s="2" t="n"/>
       <c r="L160" t="n">
@@ -11377,7 +11645,11 @@
       </c>
       <c r="G161" s="2" t="n"/>
       <c r="H161" s="2" t="n"/>
-      <c r="I161" s="2" t="n"/>
+      <c r="I161" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J161" s="2" t="n"/>
       <c r="K161" s="2" t="n"/>
       <c r="L161" t="n">
@@ -12349,7 +12621,11 @@
       </c>
       <c r="G176" s="2" t="n"/>
       <c r="H176" s="2" t="n"/>
-      <c r="I176" s="2" t="n"/>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J176" s="2" t="n"/>
       <c r="K176" s="2" t="n"/>
       <c r="L176" t="n">
@@ -12412,7 +12688,11 @@
       </c>
       <c r="G177" s="2" t="n"/>
       <c r="H177" s="2" t="n"/>
-      <c r="I177" s="2" t="n"/>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J177" s="2" t="n"/>
       <c r="K177" s="2" t="n"/>
       <c r="L177" t="n">
@@ -12475,7 +12755,11 @@
       </c>
       <c r="G178" s="2" t="n"/>
       <c r="H178" s="2" t="n"/>
-      <c r="I178" s="2" t="n"/>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J178" s="2" t="n"/>
       <c r="K178" s="2" t="n"/>
       <c r="L178" t="n">
@@ -12538,7 +12822,11 @@
       </c>
       <c r="G179" s="2" t="n"/>
       <c r="H179" s="2" t="n"/>
-      <c r="I179" s="2" t="n"/>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J179" s="2" t="n"/>
       <c r="K179" s="2" t="n"/>
       <c r="L179" t="n">
@@ -12601,7 +12889,11 @@
       </c>
       <c r="G180" s="2" t="n"/>
       <c r="H180" s="2" t="n"/>
-      <c r="I180" s="2" t="n"/>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J180" s="2" t="n"/>
       <c r="K180" s="2" t="n"/>
       <c r="L180" t="n">
@@ -12991,7 +13283,11 @@
       </c>
       <c r="G185" s="2" t="n"/>
       <c r="H185" s="2" t="n"/>
-      <c r="I185" s="2" t="n"/>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J185" s="2" t="n"/>
       <c r="K185" s="2" t="n"/>
       <c r="L185" t="n">
@@ -13054,7 +13350,11 @@
       </c>
       <c r="G186" s="2" t="n"/>
       <c r="H186" s="2" t="n"/>
-      <c r="I186" s="2" t="n"/>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J186" s="2" t="n"/>
       <c r="K186" s="2" t="n"/>
       <c r="L186" t="n">
@@ -13117,7 +13417,11 @@
       </c>
       <c r="G187" s="2" t="n"/>
       <c r="H187" s="2" t="n"/>
-      <c r="I187" s="2" t="n"/>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J187" s="2" t="n"/>
       <c r="K187" s="2" t="n"/>
       <c r="L187" t="n">
@@ -13180,7 +13484,11 @@
       </c>
       <c r="G188" s="2" t="n"/>
       <c r="H188" s="2" t="n"/>
-      <c r="I188" s="2" t="n"/>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J188" s="2" t="n"/>
       <c r="K188" s="2" t="n"/>
       <c r="L188" t="n">
@@ -13243,7 +13551,11 @@
       </c>
       <c r="G189" s="2" t="n"/>
       <c r="H189" s="2" t="n"/>
-      <c r="I189" s="2" t="n"/>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J189" s="2" t="n"/>
       <c r="K189" s="2" t="n"/>
       <c r="L189" t="n">
@@ -13807,7 +14119,11 @@
       </c>
       <c r="G196" s="2" t="n"/>
       <c r="H196" s="2" t="n"/>
-      <c r="I196" s="2" t="n"/>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J196" s="2" t="n"/>
       <c r="K196" s="2" t="n"/>
       <c r="L196" t="n">
@@ -13870,7 +14186,11 @@
       </c>
       <c r="G197" s="2" t="n"/>
       <c r="H197" s="2" t="n"/>
-      <c r="I197" s="2" t="n"/>
+      <c r="I197" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J197" s="2" t="n"/>
       <c r="K197" s="2" t="n"/>
       <c r="L197" t="n">
@@ -13933,7 +14253,11 @@
       </c>
       <c r="G198" s="2" t="n"/>
       <c r="H198" s="2" t="n"/>
-      <c r="I198" s="2" t="n"/>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J198" s="2" t="n"/>
       <c r="K198" s="2" t="n"/>
       <c r="L198" t="n">
@@ -13984,21 +14308,31 @@
           <t>ASF182</t>
         </is>
       </c>
-      <c r="E199" s="2" t="inlineStr">
+      <c r="E199" t="inlineStr">
         <is>
           <t>ASF182MM</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr">
+      <c r="F199" t="inlineStr">
         <is>
           <t>ASF182MM</t>
         </is>
       </c>
-      <c r="G199" s="2" t="n"/>
-      <c r="H199" s="2" t="n"/>
-      <c r="I199" s="2" t="n"/>
-      <c r="J199" s="2" t="n"/>
-      <c r="K199" s="2" t="n"/>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>SANDALIA</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L199" t="n">
         <v>64.34999999999999</v>
       </c>
@@ -14290,7 +14624,11 @@
       </c>
       <c r="G203" s="2" t="n"/>
       <c r="H203" s="2" t="n"/>
-      <c r="I203" s="2" t="n"/>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J203" s="2" t="n"/>
       <c r="K203" s="2" t="n"/>
       <c r="L203" t="n">
@@ -14353,7 +14691,11 @@
       </c>
       <c r="G204" s="2" t="n"/>
       <c r="H204" s="2" t="n"/>
-      <c r="I204" s="2" t="n"/>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J204" s="2" t="n"/>
       <c r="K204" s="2" t="n"/>
       <c r="L204" t="n">
@@ -14416,7 +14758,11 @@
       </c>
       <c r="G205" s="2" t="n"/>
       <c r="H205" s="2" t="n"/>
-      <c r="I205" s="2" t="n"/>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J205" s="2" t="n"/>
       <c r="K205" s="2" t="n"/>
       <c r="L205" t="n">
@@ -14479,7 +14825,11 @@
       </c>
       <c r="G206" s="2" t="n"/>
       <c r="H206" s="2" t="n"/>
-      <c r="I206" s="2" t="n"/>
+      <c r="I206" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J206" s="2" t="n"/>
       <c r="K206" s="2" t="n"/>
       <c r="L206" t="n">
@@ -14542,7 +14892,11 @@
       </c>
       <c r="G207" s="2" t="n"/>
       <c r="H207" s="2" t="n"/>
-      <c r="I207" s="2" t="n"/>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J207" s="2" t="n"/>
       <c r="K207" s="2" t="n"/>
       <c r="L207" t="n">
@@ -14605,7 +14959,11 @@
       </c>
       <c r="G208" s="2" t="n"/>
       <c r="H208" s="2" t="n"/>
-      <c r="I208" s="2" t="n"/>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J208" s="2" t="n"/>
       <c r="K208" s="2" t="n"/>
       <c r="L208" t="n">
@@ -14967,7 +15325,11 @@
       </c>
       <c r="G214" s="2" t="n"/>
       <c r="H214" s="2" t="n"/>
-      <c r="I214" s="2" t="n"/>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J214" s="2" t="n"/>
       <c r="K214" s="2" t="n"/>
       <c r="L214" t="n">
@@ -15030,7 +15392,11 @@
       </c>
       <c r="G215" s="2" t="n"/>
       <c r="H215" s="2" t="n"/>
-      <c r="I215" s="2" t="n"/>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J215" s="2" t="n"/>
       <c r="K215" s="2" t="n"/>
       <c r="L215" t="n">
@@ -15093,7 +15459,11 @@
       </c>
       <c r="G216" s="2" t="n"/>
       <c r="H216" s="2" t="n"/>
-      <c r="I216" s="2" t="n"/>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J216" s="2" t="n"/>
       <c r="K216" s="2" t="n"/>
       <c r="L216" t="n">
@@ -15156,7 +15526,11 @@
       </c>
       <c r="G217" s="2" t="n"/>
       <c r="H217" s="2" t="n"/>
-      <c r="I217" s="2" t="n"/>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J217" s="2" t="n"/>
       <c r="K217" s="2" t="n"/>
       <c r="L217" t="n">
@@ -15219,7 +15593,11 @@
       </c>
       <c r="G218" s="2" t="n"/>
       <c r="H218" s="2" t="n"/>
-      <c r="I218" s="2" t="n"/>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J218" s="2" t="n"/>
       <c r="K218" s="2" t="n"/>
       <c r="L218" t="n">
@@ -15363,7 +15741,11 @@
       </c>
       <c r="G220" s="2" t="n"/>
       <c r="H220" s="2" t="n"/>
-      <c r="I220" s="2" t="n"/>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J220" s="2" t="n"/>
       <c r="K220" s="2" t="n"/>
       <c r="L220" t="n">
@@ -15426,7 +15808,11 @@
       </c>
       <c r="G221" s="2" t="n"/>
       <c r="H221" s="2" t="n"/>
-      <c r="I221" s="2" t="n"/>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J221" s="2" t="n"/>
       <c r="K221" s="2" t="n"/>
       <c r="L221" t="n">
@@ -15489,7 +15875,11 @@
       </c>
       <c r="G222" s="2" t="n"/>
       <c r="H222" s="2" t="n"/>
-      <c r="I222" s="2" t="n"/>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J222" s="2" t="n"/>
       <c r="K222" s="2" t="n"/>
       <c r="L222" t="n">
@@ -15552,7 +15942,11 @@
       </c>
       <c r="G223" s="2" t="n"/>
       <c r="H223" s="2" t="n"/>
-      <c r="I223" s="2" t="n"/>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J223" s="2" t="n"/>
       <c r="K223" s="2" t="n"/>
       <c r="L223" t="n">
@@ -16135,7 +16529,11 @@
       </c>
       <c r="G232" s="2" t="n"/>
       <c r="H232" s="2" t="n"/>
-      <c r="I232" s="2" t="n"/>
+      <c r="I232" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J232" s="2" t="n"/>
       <c r="K232" s="2" t="n"/>
       <c r="L232" t="n">
@@ -16241,7 +16639,11 @@
       </c>
       <c r="G234" s="2" t="n"/>
       <c r="H234" s="2" t="n"/>
-      <c r="I234" s="2" t="n"/>
+      <c r="I234" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J234" s="2" t="n"/>
       <c r="K234" s="2" t="n"/>
       <c r="L234" t="n">
@@ -16307,7 +16709,11 @@
       </c>
       <c r="G235" s="2" t="n"/>
       <c r="H235" s="2" t="n"/>
-      <c r="I235" s="2" t="n"/>
+      <c r="I235" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J235" s="2" t="n"/>
       <c r="K235" s="2" t="n"/>
       <c r="L235" t="n">
@@ -16370,7 +16776,11 @@
       </c>
       <c r="G236" s="2" t="n"/>
       <c r="H236" s="2" t="n"/>
-      <c r="I236" s="2" t="n"/>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J236" s="2" t="n"/>
       <c r="K236" s="2" t="n"/>
       <c r="L236" t="n">
@@ -17067,7 +17477,11 @@
       </c>
       <c r="G246" s="2" t="n"/>
       <c r="H246" s="2" t="n"/>
-      <c r="I246" s="2" t="n"/>
+      <c r="I246" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J246" s="2" t="n"/>
       <c r="K246" s="2" t="n"/>
       <c r="L246" t="n">
@@ -17130,7 +17544,11 @@
       </c>
       <c r="G247" s="2" t="n"/>
       <c r="H247" s="2" t="n"/>
-      <c r="I247" s="2" t="n"/>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J247" s="2" t="n"/>
       <c r="K247" s="2" t="n"/>
       <c r="L247" t="n">
@@ -17193,7 +17611,11 @@
       </c>
       <c r="G248" s="2" t="n"/>
       <c r="H248" s="2" t="n"/>
-      <c r="I248" s="2" t="n"/>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J248" s="2" t="n"/>
       <c r="K248" s="2" t="n"/>
       <c r="L248" t="n">
@@ -17244,21 +17666,31 @@
           <t>ASF182</t>
         </is>
       </c>
-      <c r="E249" s="2" t="inlineStr">
+      <c r="E249" t="inlineStr">
         <is>
           <t>ASF182MM</t>
         </is>
       </c>
-      <c r="F249" s="2" t="inlineStr">
+      <c r="F249" t="inlineStr">
         <is>
           <t>ASF182MM</t>
         </is>
       </c>
-      <c r="G249" s="2" t="n"/>
-      <c r="H249" s="2" t="n"/>
-      <c r="I249" s="2" t="n"/>
-      <c r="J249" s="2" t="n"/>
-      <c r="K249" s="2" t="n"/>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>SANDALIA</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L249" t="n">
         <v>64.34999999999999</v>
       </c>
@@ -18069,7 +18501,11 @@
       </c>
       <c r="G260" s="2" t="n"/>
       <c r="H260" s="2" t="n"/>
-      <c r="I260" s="2" t="n"/>
+      <c r="I260" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J260" s="2" t="n"/>
       <c r="K260" s="2" t="n"/>
       <c r="L260" t="n">
@@ -18132,7 +18568,11 @@
       </c>
       <c r="G261" s="2" t="n"/>
       <c r="H261" s="2" t="n"/>
-      <c r="I261" s="2" t="n"/>
+      <c r="I261" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J261" s="2" t="n"/>
       <c r="K261" s="2" t="n"/>
       <c r="L261" t="n">
@@ -18357,7 +18797,11 @@
       </c>
       <c r="G264" s="2" t="n"/>
       <c r="H264" s="2" t="n"/>
-      <c r="I264" s="2" t="n"/>
+      <c r="I264" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J264" s="2" t="n"/>
       <c r="K264" s="2" t="n"/>
       <c r="L264" t="n">
@@ -18463,7 +18907,11 @@
       </c>
       <c r="G266" s="2" t="n"/>
       <c r="H266" s="2" t="n"/>
-      <c r="I266" s="2" t="n"/>
+      <c r="I266" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J266" s="2" t="n"/>
       <c r="K266" s="2" t="n"/>
       <c r="L266" t="n">
@@ -18511,7 +18959,11 @@
       </c>
       <c r="G267" s="2" t="n"/>
       <c r="H267" s="2" t="n"/>
-      <c r="I267" s="2" t="n"/>
+      <c r="I267" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J267" s="2" t="n"/>
       <c r="K267" s="2" t="n"/>
       <c r="L267" t="n">
@@ -18559,7 +19011,11 @@
       </c>
       <c r="G268" s="2" t="n"/>
       <c r="H268" s="2" t="n"/>
-      <c r="I268" s="2" t="n"/>
+      <c r="I268" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J268" s="2" t="n"/>
       <c r="K268" s="2" t="n"/>
       <c r="L268" t="n">
@@ -18871,7 +19327,11 @@
       </c>
       <c r="G273" s="2" t="n"/>
       <c r="H273" s="2" t="n"/>
-      <c r="I273" s="2" t="n"/>
+      <c r="I273" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J273" s="2" t="n"/>
       <c r="K273" s="2" t="n"/>
       <c r="L273" t="n">
@@ -18919,7 +19379,11 @@
       </c>
       <c r="G274" s="2" t="n"/>
       <c r="H274" s="2" t="n"/>
-      <c r="I274" s="2" t="n"/>
+      <c r="I274" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J274" s="2" t="n"/>
       <c r="K274" s="2" t="n"/>
       <c r="L274" t="n">
@@ -18967,7 +19431,11 @@
       </c>
       <c r="G275" s="2" t="n"/>
       <c r="H275" s="2" t="n"/>
-      <c r="I275" s="2" t="n"/>
+      <c r="I275" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J275" s="2" t="n"/>
       <c r="K275" s="2" t="n"/>
       <c r="L275" t="n">
@@ -19147,7 +19615,11 @@
       </c>
       <c r="G278" s="2" t="n"/>
       <c r="H278" s="2" t="n"/>
-      <c r="I278" s="2" t="n"/>
+      <c r="I278" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J278" s="2" t="n"/>
       <c r="K278" s="2" t="n"/>
       <c r="L278" t="n">
@@ -19210,7 +19682,11 @@
       </c>
       <c r="G279" s="2" t="n"/>
       <c r="H279" s="2" t="n"/>
-      <c r="I279" s="2" t="n"/>
+      <c r="I279" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J279" s="2" t="n"/>
       <c r="K279" s="2" t="n"/>
       <c r="L279" t="n">
@@ -19273,7 +19749,11 @@
       </c>
       <c r="G280" s="2" t="n"/>
       <c r="H280" s="2" t="n"/>
-      <c r="I280" s="2" t="n"/>
+      <c r="I280" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J280" s="2" t="n"/>
       <c r="K280" s="2" t="n"/>
       <c r="L280" t="n">
@@ -19405,21 +19885,31 @@
           <t>WSC330</t>
         </is>
       </c>
-      <c r="E282" s="2" t="inlineStr">
+      <c r="E282" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="F282" s="2" t="inlineStr">
+      <c r="F282" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="G282" s="2" t="n"/>
-      <c r="H282" s="2" t="n"/>
-      <c r="I282" s="2" t="n"/>
-      <c r="J282" s="2" t="n"/>
-      <c r="K282" s="2" t="n"/>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L282" t="n">
         <v>68.31999999999999</v>
       </c>
@@ -20002,7 +20492,11 @@
       </c>
       <c r="G290" s="2" t="n"/>
       <c r="H290" s="2" t="n"/>
-      <c r="I290" s="2" t="n"/>
+      <c r="I290" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J290" s="2" t="n"/>
       <c r="K290" s="2" t="n"/>
       <c r="L290" t="n">
@@ -20146,7 +20640,11 @@
       </c>
       <c r="G292" s="2" t="n"/>
       <c r="H292" s="2" t="n"/>
-      <c r="I292" s="2" t="n"/>
+      <c r="I292" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J292" s="2" t="n"/>
       <c r="K292" s="2" t="n"/>
       <c r="L292" t="n">
@@ -20209,7 +20707,11 @@
       </c>
       <c r="G293" s="2" t="n"/>
       <c r="H293" s="2" t="n"/>
-      <c r="I293" s="2" t="n"/>
+      <c r="I293" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J293" s="2" t="n"/>
       <c r="K293" s="2" t="n"/>
       <c r="L293" t="n">
@@ -20272,7 +20774,11 @@
       </c>
       <c r="G294" s="2" t="n"/>
       <c r="H294" s="2" t="n"/>
-      <c r="I294" s="2" t="n"/>
+      <c r="I294" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J294" s="2" t="n"/>
       <c r="K294" s="2" t="n"/>
       <c r="L294" t="n">
@@ -20335,7 +20841,11 @@
       </c>
       <c r="G295" s="2" t="n"/>
       <c r="H295" s="2" t="n"/>
-      <c r="I295" s="2" t="n"/>
+      <c r="I295" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J295" s="2" t="n"/>
       <c r="K295" s="2" t="n"/>
       <c r="L295" t="n">
@@ -20530,7 +21040,11 @@
       </c>
       <c r="G298" s="2" t="n"/>
       <c r="H298" s="2" t="n"/>
-      <c r="I298" s="2" t="n"/>
+      <c r="I298" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J298" s="2" t="n"/>
       <c r="K298" s="2" t="n"/>
       <c r="L298" t="n">
@@ -20644,7 +21158,11 @@
       </c>
       <c r="G300" s="2" t="n"/>
       <c r="H300" s="2" t="n"/>
-      <c r="I300" s="2" t="n"/>
+      <c r="I300" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J300" s="2" t="n"/>
       <c r="K300" s="2" t="n"/>
       <c r="L300" t="n">
@@ -20695,21 +21213,31 @@
           <t>ASF182</t>
         </is>
       </c>
-      <c r="E301" s="2" t="inlineStr">
+      <c r="E301" t="inlineStr">
         <is>
           <t>ASF182MM</t>
         </is>
       </c>
-      <c r="F301" s="2" t="inlineStr">
+      <c r="F301" t="inlineStr">
         <is>
           <t>ASF182MM</t>
         </is>
       </c>
-      <c r="G301" s="2" t="n"/>
-      <c r="H301" s="2" t="n"/>
-      <c r="I301" s="2" t="n"/>
-      <c r="J301" s="2" t="n"/>
-      <c r="K301" s="2" t="n"/>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>SANDALIA</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L301" t="n">
         <v>64.34999999999999</v>
       </c>
@@ -20908,21 +21436,31 @@
           <t>WSC330</t>
         </is>
       </c>
-      <c r="E304" s="2" t="inlineStr">
+      <c r="E304" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="F304" s="2" t="inlineStr">
+      <c r="F304" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="G304" s="2" t="n"/>
-      <c r="H304" s="2" t="n"/>
-      <c r="I304" s="2" t="n"/>
-      <c r="J304" s="2" t="n"/>
-      <c r="K304" s="2" t="n"/>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L304" t="n">
         <v>68.31999999999999</v>
       </c>
@@ -21226,7 +21764,11 @@
       </c>
       <c r="G308" s="2" t="n"/>
       <c r="H308" s="2" t="n"/>
-      <c r="I308" s="2" t="n"/>
+      <c r="I308" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J308" s="2" t="n"/>
       <c r="K308" s="2" t="n"/>
       <c r="L308" t="n">
@@ -21289,7 +21831,11 @@
       </c>
       <c r="G309" s="2" t="n"/>
       <c r="H309" s="2" t="n"/>
-      <c r="I309" s="2" t="n"/>
+      <c r="I309" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J309" s="2" t="n"/>
       <c r="K309" s="2" t="n"/>
       <c r="L309" t="n">
@@ -21352,7 +21898,11 @@
       </c>
       <c r="G310" s="2" t="n"/>
       <c r="H310" s="2" t="n"/>
-      <c r="I310" s="2" t="n"/>
+      <c r="I310" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J310" s="2" t="n"/>
       <c r="K310" s="2" t="n"/>
       <c r="L310" t="n">
@@ -21574,7 +22124,11 @@
       </c>
       <c r="G313" s="2" t="n"/>
       <c r="H313" s="2" t="n"/>
-      <c r="I313" s="2" t="n"/>
+      <c r="I313" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J313" s="2" t="n"/>
       <c r="K313" s="2" t="n"/>
       <c r="L313" t="n">
@@ -21637,7 +22191,11 @@
       </c>
       <c r="G314" s="2" t="n"/>
       <c r="H314" s="2" t="n"/>
-      <c r="I314" s="2" t="n"/>
+      <c r="I314" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J314" s="2" t="n"/>
       <c r="K314" s="2" t="n"/>
       <c r="L314" t="n">
@@ -21700,7 +22258,11 @@
       </c>
       <c r="G315" s="2" t="n"/>
       <c r="H315" s="2" t="n"/>
-      <c r="I315" s="2" t="n"/>
+      <c r="I315" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J315" s="2" t="n"/>
       <c r="K315" s="2" t="n"/>
       <c r="L315" t="n">
@@ -21763,7 +22325,11 @@
       </c>
       <c r="G316" s="2" t="n"/>
       <c r="H316" s="2" t="n"/>
-      <c r="I316" s="2" t="n"/>
+      <c r="I316" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J316" s="2" t="n"/>
       <c r="K316" s="2" t="n"/>
       <c r="L316" t="n">
@@ -21826,7 +22392,11 @@
       </c>
       <c r="G317" s="2" t="n"/>
       <c r="H317" s="2" t="n"/>
-      <c r="I317" s="2" t="n"/>
+      <c r="I317" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J317" s="2" t="n"/>
       <c r="K317" s="2" t="n"/>
       <c r="L317" t="n">
@@ -22219,7 +22789,11 @@
       </c>
       <c r="G323" s="2" t="n"/>
       <c r="H323" s="2" t="n"/>
-      <c r="I323" s="2" t="n"/>
+      <c r="I323" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J323" s="2" t="n"/>
       <c r="K323" s="2" t="n"/>
       <c r="L323" t="n">
@@ -22285,7 +22859,11 @@
       </c>
       <c r="G324" s="2" t="n"/>
       <c r="H324" s="2" t="n"/>
-      <c r="I324" s="2" t="n"/>
+      <c r="I324" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J324" s="2" t="n"/>
       <c r="K324" s="2" t="n"/>
       <c r="L324" t="n">
@@ -22351,7 +22929,11 @@
       </c>
       <c r="G325" s="2" t="n"/>
       <c r="H325" s="2" t="n"/>
-      <c r="I325" s="2" t="n"/>
+      <c r="I325" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J325" s="2" t="n"/>
       <c r="K325" s="2" t="n"/>
       <c r="L325" t="n">
@@ -22414,7 +22996,11 @@
       </c>
       <c r="G326" s="2" t="n"/>
       <c r="H326" s="2" t="n"/>
-      <c r="I326" s="2" t="n"/>
+      <c r="I326" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J326" s="2" t="n"/>
       <c r="K326" s="2" t="n"/>
       <c r="L326" t="n">
@@ -22477,7 +23063,11 @@
       </c>
       <c r="G327" s="2" t="n"/>
       <c r="H327" s="2" t="n"/>
-      <c r="I327" s="2" t="n"/>
+      <c r="I327" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J327" s="2" t="n"/>
       <c r="K327" s="2" t="n"/>
       <c r="L327" t="n">
@@ -22540,7 +23130,11 @@
       </c>
       <c r="G328" s="2" t="n"/>
       <c r="H328" s="2" t="n"/>
-      <c r="I328" s="2" t="n"/>
+      <c r="I328" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J328" s="2" t="n"/>
       <c r="K328" s="2" t="n"/>
       <c r="L328" t="n">
@@ -22603,7 +23197,11 @@
       </c>
       <c r="G329" s="2" t="n"/>
       <c r="H329" s="2" t="n"/>
-      <c r="I329" s="2" t="n"/>
+      <c r="I329" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J329" s="2" t="n"/>
       <c r="K329" s="2" t="n"/>
       <c r="L329" t="n">
@@ -22666,7 +23264,11 @@
       </c>
       <c r="G330" s="2" t="n"/>
       <c r="H330" s="2" t="n"/>
-      <c r="I330" s="2" t="n"/>
+      <c r="I330" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J330" s="2" t="n"/>
       <c r="K330" s="2" t="n"/>
       <c r="L330" t="n">
@@ -23365,21 +23967,39 @@
           <t>SAF126</t>
         </is>
       </c>
-      <c r="E340" s="2" t="inlineStr">
+      <c r="E340" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="F340" s="2" t="inlineStr">
+      <c r="F340" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="G340" s="2" t="n"/>
-      <c r="H340" s="2" t="n"/>
-      <c r="I340" s="2" t="n"/>
-      <c r="J340" s="2" t="n"/>
-      <c r="K340" s="2" t="n"/>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
+      <c r="J340" t="n">
+        <v>249.9</v>
+      </c>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="L340" t="n">
         <v>135.3</v>
       </c>
@@ -23443,7 +24063,11 @@
       </c>
       <c r="G341" s="2" t="n"/>
       <c r="H341" s="2" t="n"/>
-      <c r="I341" s="2" t="n"/>
+      <c r="I341" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J341" s="2" t="n"/>
       <c r="K341" s="2" t="n"/>
       <c r="L341" t="n">
@@ -23668,7 +24292,11 @@
       </c>
       <c r="G344" s="2" t="n"/>
       <c r="H344" s="2" t="n"/>
-      <c r="I344" s="2" t="n"/>
+      <c r="I344" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J344" s="2" t="n"/>
       <c r="K344" s="2" t="n"/>
       <c r="L344" t="n">
@@ -23716,7 +24344,11 @@
       </c>
       <c r="G345" s="2" t="n"/>
       <c r="H345" s="2" t="n"/>
-      <c r="I345" s="2" t="n"/>
+      <c r="I345" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J345" s="2" t="n"/>
       <c r="K345" s="2" t="n"/>
       <c r="L345" t="n">
@@ -23764,7 +24396,11 @@
       </c>
       <c r="G346" s="2" t="n"/>
       <c r="H346" s="2" t="n"/>
-      <c r="I346" s="2" t="n"/>
+      <c r="I346" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J346" s="2" t="n"/>
       <c r="K346" s="2" t="n"/>
       <c r="L346" t="n">
@@ -23944,7 +24580,11 @@
       </c>
       <c r="G349" s="2" t="n"/>
       <c r="H349" s="2" t="n"/>
-      <c r="I349" s="2" t="n"/>
+      <c r="I349" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J349" s="2" t="n"/>
       <c r="K349" s="2" t="n"/>
       <c r="L349" t="n">
@@ -23992,7 +24632,11 @@
       </c>
       <c r="G350" s="2" t="n"/>
       <c r="H350" s="2" t="n"/>
-      <c r="I350" s="2" t="n"/>
+      <c r="I350" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J350" s="2" t="n"/>
       <c r="K350" s="2" t="n"/>
       <c r="L350" t="n">
@@ -24040,7 +24684,11 @@
       </c>
       <c r="G351" s="2" t="n"/>
       <c r="H351" s="2" t="n"/>
-      <c r="I351" s="2" t="n"/>
+      <c r="I351" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J351" s="2" t="n"/>
       <c r="K351" s="2" t="n"/>
       <c r="L351" t="n">
@@ -24484,7 +25132,11 @@
       </c>
       <c r="G358" s="2" t="n"/>
       <c r="H358" s="2" t="n"/>
-      <c r="I358" s="2" t="n"/>
+      <c r="I358" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J358" s="2" t="n"/>
       <c r="K358" s="2" t="n"/>
       <c r="L358" t="n">
@@ -24628,7 +25280,11 @@
       </c>
       <c r="G360" s="2" t="n"/>
       <c r="H360" s="2" t="n"/>
-      <c r="I360" s="2" t="n"/>
+      <c r="I360" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J360" s="2" t="n"/>
       <c r="K360" s="2" t="n"/>
       <c r="L360" t="n">
@@ -24691,7 +25347,11 @@
       </c>
       <c r="G361" s="2" t="n"/>
       <c r="H361" s="2" t="n"/>
-      <c r="I361" s="2" t="n"/>
+      <c r="I361" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J361" s="2" t="n"/>
       <c r="K361" s="2" t="n"/>
       <c r="L361" t="n">
@@ -24754,7 +25414,11 @@
       </c>
       <c r="G362" s="2" t="n"/>
       <c r="H362" s="2" t="n"/>
-      <c r="I362" s="2" t="n"/>
+      <c r="I362" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J362" s="2" t="n"/>
       <c r="K362" s="2" t="n"/>
       <c r="L362" t="n">
@@ -25060,7 +25724,11 @@
       </c>
       <c r="G366" s="2" t="n"/>
       <c r="H366" s="2" t="n"/>
-      <c r="I366" s="2" t="n"/>
+      <c r="I366" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J366" s="2" t="n"/>
       <c r="K366" s="2" t="n"/>
       <c r="L366" t="n">
@@ -25123,7 +25791,11 @@
       </c>
       <c r="G367" s="2" t="n"/>
       <c r="H367" s="2" t="n"/>
-      <c r="I367" s="2" t="n"/>
+      <c r="I367" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J367" s="2" t="n"/>
       <c r="K367" s="2" t="n"/>
       <c r="L367" t="n">
@@ -25186,7 +25858,11 @@
       </c>
       <c r="G368" s="2" t="n"/>
       <c r="H368" s="2" t="n"/>
-      <c r="I368" s="2" t="n"/>
+      <c r="I368" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J368" s="2" t="n"/>
       <c r="K368" s="2" t="n"/>
       <c r="L368" t="n">
@@ -25687,7 +26363,11 @@
       </c>
       <c r="G375" s="2" t="n"/>
       <c r="H375" s="2" t="n"/>
-      <c r="I375" s="2" t="n"/>
+      <c r="I375" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J375" s="2" t="n"/>
       <c r="K375" s="2" t="n"/>
       <c r="L375" t="n">
@@ -26212,7 +26892,11 @@
       </c>
       <c r="G383" s="2" t="n"/>
       <c r="H383" s="2" t="n"/>
-      <c r="I383" s="2" t="n"/>
+      <c r="I383" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J383" s="2" t="n"/>
       <c r="K383" s="2" t="n"/>
       <c r="L383" t="n">
@@ -26356,7 +27040,11 @@
       </c>
       <c r="G385" s="2" t="n"/>
       <c r="H385" s="2" t="n"/>
-      <c r="I385" s="2" t="n"/>
+      <c r="I385" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J385" s="2" t="n"/>
       <c r="K385" s="2" t="n"/>
       <c r="L385" t="n">
@@ -26419,7 +27107,11 @@
       </c>
       <c r="G386" s="2" t="n"/>
       <c r="H386" s="2" t="n"/>
-      <c r="I386" s="2" t="n"/>
+      <c r="I386" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J386" s="2" t="n"/>
       <c r="K386" s="2" t="n"/>
       <c r="L386" t="n">
@@ -26470,21 +27162,31 @@
           <t>WSC330</t>
         </is>
       </c>
-      <c r="E387" s="2" t="inlineStr">
+      <c r="E387" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="F387" s="2" t="inlineStr">
+      <c r="F387" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="G387" s="2" t="n"/>
-      <c r="H387" s="2" t="n"/>
-      <c r="I387" s="2" t="n"/>
-      <c r="J387" s="2" t="n"/>
-      <c r="K387" s="2" t="n"/>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L387" t="n">
         <v>68.31999999999999</v>
       </c>
@@ -26707,7 +27409,11 @@
       </c>
       <c r="G390" s="2" t="n"/>
       <c r="H390" s="2" t="n"/>
-      <c r="I390" s="2" t="n"/>
+      <c r="I390" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J390" s="2" t="n"/>
       <c r="K390" s="2" t="n"/>
       <c r="L390" t="n">
@@ -26755,7 +27461,11 @@
       </c>
       <c r="G391" s="2" t="n"/>
       <c r="H391" s="2" t="n"/>
-      <c r="I391" s="2" t="n"/>
+      <c r="I391" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J391" s="2" t="n"/>
       <c r="K391" s="2" t="n"/>
       <c r="L391" t="n">
@@ -26803,7 +27513,11 @@
       </c>
       <c r="G392" s="2" t="n"/>
       <c r="H392" s="2" t="n"/>
-      <c r="I392" s="2" t="n"/>
+      <c r="I392" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J392" s="2" t="n"/>
       <c r="K392" s="2" t="n"/>
       <c r="L392" t="n">
@@ -26851,7 +27565,11 @@
       </c>
       <c r="G393" s="2" t="n"/>
       <c r="H393" s="2" t="n"/>
-      <c r="I393" s="2" t="n"/>
+      <c r="I393" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J393" s="2" t="n"/>
       <c r="K393" s="2" t="n"/>
       <c r="L393" t="n">
@@ -26899,7 +27617,11 @@
       </c>
       <c r="G394" s="2" t="n"/>
       <c r="H394" s="2" t="n"/>
-      <c r="I394" s="2" t="n"/>
+      <c r="I394" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J394" s="2" t="n"/>
       <c r="K394" s="2" t="n"/>
       <c r="L394" t="n">
@@ -27079,7 +27801,11 @@
       </c>
       <c r="G397" s="2" t="n"/>
       <c r="H397" s="2" t="n"/>
-      <c r="I397" s="2" t="n"/>
+      <c r="I397" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J397" s="2" t="n"/>
       <c r="K397" s="2" t="n"/>
       <c r="L397" t="n">
@@ -27127,7 +27853,11 @@
       </c>
       <c r="G398" s="2" t="n"/>
       <c r="H398" s="2" t="n"/>
-      <c r="I398" s="2" t="n"/>
+      <c r="I398" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J398" s="2" t="n"/>
       <c r="K398" s="2" t="n"/>
       <c r="L398" t="n">
@@ -27175,7 +27905,11 @@
       </c>
       <c r="G399" s="2" t="n"/>
       <c r="H399" s="2" t="n"/>
-      <c r="I399" s="2" t="n"/>
+      <c r="I399" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J399" s="2" t="n"/>
       <c r="K399" s="2" t="n"/>
       <c r="L399" t="n">
@@ -27370,7 +28104,11 @@
       </c>
       <c r="G402" s="2" t="n"/>
       <c r="H402" s="2" t="n"/>
-      <c r="I402" s="2" t="n"/>
+      <c r="I402" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J402" s="2" t="n"/>
       <c r="K402" s="2" t="n"/>
       <c r="L402" t="n">
@@ -27433,7 +28171,11 @@
       </c>
       <c r="G403" s="2" t="n"/>
       <c r="H403" s="2" t="n"/>
-      <c r="I403" s="2" t="n"/>
+      <c r="I403" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J403" s="2" t="n"/>
       <c r="K403" s="2" t="n"/>
       <c r="L403" t="n">
@@ -27496,7 +28238,11 @@
       </c>
       <c r="G404" s="2" t="n"/>
       <c r="H404" s="2" t="n"/>
-      <c r="I404" s="2" t="n"/>
+      <c r="I404" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J404" s="2" t="n"/>
       <c r="K404" s="2" t="n"/>
       <c r="L404" t="n">
@@ -27559,7 +28305,11 @@
       </c>
       <c r="G405" s="2" t="n"/>
       <c r="H405" s="2" t="n"/>
-      <c r="I405" s="2" t="n"/>
+      <c r="I405" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J405" s="2" t="n"/>
       <c r="K405" s="2" t="n"/>
       <c r="L405" t="n">
@@ -27754,7 +28504,11 @@
       </c>
       <c r="G408" s="2" t="n"/>
       <c r="H408" s="2" t="n"/>
-      <c r="I408" s="2" t="n"/>
+      <c r="I408" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J408" s="2" t="n"/>
       <c r="K408" s="2" t="n"/>
       <c r="L408" t="n">
@@ -27817,7 +28571,11 @@
       </c>
       <c r="G409" s="2" t="n"/>
       <c r="H409" s="2" t="n"/>
-      <c r="I409" s="2" t="n"/>
+      <c r="I409" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J409" s="2" t="n"/>
       <c r="K409" s="2" t="n"/>
       <c r="L409" t="n">
@@ -27880,7 +28638,11 @@
       </c>
       <c r="G410" s="2" t="n"/>
       <c r="H410" s="2" t="n"/>
-      <c r="I410" s="2" t="n"/>
+      <c r="I410" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J410" s="2" t="n"/>
       <c r="K410" s="2" t="n"/>
       <c r="L410" t="n">
@@ -27943,7 +28705,11 @@
       </c>
       <c r="G411" s="2" t="n"/>
       <c r="H411" s="2" t="n"/>
-      <c r="I411" s="2" t="n"/>
+      <c r="I411" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J411" s="2" t="n"/>
       <c r="K411" s="2" t="n"/>
       <c r="L411" t="n">
@@ -28006,7 +28772,11 @@
       </c>
       <c r="G412" s="2" t="n"/>
       <c r="H412" s="2" t="n"/>
-      <c r="I412" s="2" t="n"/>
+      <c r="I412" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J412" s="2" t="n"/>
       <c r="K412" s="2" t="n"/>
       <c r="L412" t="n">
@@ -28465,7 +29235,11 @@
       </c>
       <c r="G419" s="2" t="n"/>
       <c r="H419" s="2" t="n"/>
-      <c r="I419" s="2" t="n"/>
+      <c r="I419" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J419" s="2" t="n"/>
       <c r="K419" s="2" t="n"/>
       <c r="L419" t="n">
@@ -28528,7 +29302,11 @@
       </c>
       <c r="G420" s="2" t="n"/>
       <c r="H420" s="2" t="n"/>
-      <c r="I420" s="2" t="n"/>
+      <c r="I420" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J420" s="2" t="n"/>
       <c r="K420" s="2" t="n"/>
       <c r="L420" t="n">
@@ -28591,7 +29369,11 @@
       </c>
       <c r="G421" s="2" t="n"/>
       <c r="H421" s="2" t="n"/>
-      <c r="I421" s="2" t="n"/>
+      <c r="I421" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J421" s="2" t="n"/>
       <c r="K421" s="2" t="n"/>
       <c r="L421" t="n">
@@ -28654,7 +29436,11 @@
       </c>
       <c r="G422" s="2" t="n"/>
       <c r="H422" s="2" t="n"/>
-      <c r="I422" s="2" t="n"/>
+      <c r="I422" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J422" s="2" t="n"/>
       <c r="K422" s="2" t="n"/>
       <c r="L422" t="n">
@@ -28717,7 +29503,11 @@
       </c>
       <c r="G423" s="2" t="n"/>
       <c r="H423" s="2" t="n"/>
-      <c r="I423" s="2" t="n"/>
+      <c r="I423" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J423" s="2" t="n"/>
       <c r="K423" s="2" t="n"/>
       <c r="L423" t="n">
@@ -28780,7 +29570,11 @@
       </c>
       <c r="G424" s="2" t="n"/>
       <c r="H424" s="2" t="n"/>
-      <c r="I424" s="2" t="n"/>
+      <c r="I424" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J424" s="2" t="n"/>
       <c r="K424" s="2" t="n"/>
       <c r="L424" t="n">
@@ -29254,7 +30048,11 @@
       </c>
       <c r="G431" s="2" t="n"/>
       <c r="H431" s="2" t="n"/>
-      <c r="I431" s="2" t="n"/>
+      <c r="I431" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J431" s="2" t="n"/>
       <c r="K431" s="2" t="n"/>
       <c r="L431" t="n">
@@ -29317,7 +30115,11 @@
       </c>
       <c r="G432" s="2" t="n"/>
       <c r="H432" s="2" t="n"/>
-      <c r="I432" s="2" t="n"/>
+      <c r="I432" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J432" s="2" t="n"/>
       <c r="K432" s="2" t="n"/>
       <c r="L432" t="n">
@@ -29380,7 +30182,11 @@
       </c>
       <c r="G433" s="2" t="n"/>
       <c r="H433" s="2" t="n"/>
-      <c r="I433" s="2" t="n"/>
+      <c r="I433" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J433" s="2" t="n"/>
       <c r="K433" s="2" t="n"/>
       <c r="L433" t="n">
@@ -29443,7 +30249,11 @@
       </c>
       <c r="G434" s="2" t="n"/>
       <c r="H434" s="2" t="n"/>
-      <c r="I434" s="2" t="n"/>
+      <c r="I434" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J434" s="2" t="n"/>
       <c r="K434" s="2" t="n"/>
       <c r="L434" t="n">
@@ -29506,7 +30316,11 @@
       </c>
       <c r="G435" s="2" t="n"/>
       <c r="H435" s="2" t="n"/>
-      <c r="I435" s="2" t="n"/>
+      <c r="I435" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J435" s="2" t="n"/>
       <c r="K435" s="2" t="n"/>
       <c r="L435" t="n">
@@ -29569,7 +30383,11 @@
       </c>
       <c r="G436" s="2" t="n"/>
       <c r="H436" s="2" t="n"/>
-      <c r="I436" s="2" t="n"/>
+      <c r="I436" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J436" s="2" t="n"/>
       <c r="K436" s="2" t="n"/>
       <c r="L436" t="n">
@@ -29845,7 +30663,11 @@
       </c>
       <c r="G440" s="2" t="n"/>
       <c r="H440" s="2" t="n"/>
-      <c r="I440" s="2" t="n"/>
+      <c r="I440" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J440" s="2" t="n"/>
       <c r="K440" s="2" t="n"/>
       <c r="L440" t="n">
@@ -29908,7 +30730,11 @@
       </c>
       <c r="G441" s="2" t="n"/>
       <c r="H441" s="2" t="n"/>
-      <c r="I441" s="2" t="n"/>
+      <c r="I441" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J441" s="2" t="n"/>
       <c r="K441" s="2" t="n"/>
       <c r="L441" t="n">
@@ -29959,21 +30785,31 @@
           <t>ASF182</t>
         </is>
       </c>
-      <c r="E442" s="2" t="inlineStr">
+      <c r="E442" t="inlineStr">
         <is>
           <t>ASF182MM</t>
         </is>
       </c>
-      <c r="F442" s="2" t="inlineStr">
+      <c r="F442" t="inlineStr">
         <is>
           <t>ASF182MM</t>
         </is>
       </c>
-      <c r="G442" s="2" t="n"/>
-      <c r="H442" s="2" t="n"/>
-      <c r="I442" s="2" t="n"/>
-      <c r="J442" s="2" t="n"/>
-      <c r="K442" s="2" t="n"/>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>SANDALIA</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L442" t="n">
         <v>64.34999999999999</v>
       </c>
@@ -30577,7 +31413,11 @@
       </c>
       <c r="G451" s="2" t="n"/>
       <c r="H451" s="2" t="n"/>
-      <c r="I451" s="2" t="n"/>
+      <c r="I451" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J451" s="2" t="n"/>
       <c r="K451" s="2" t="n"/>
       <c r="L451" t="n">
@@ -30709,21 +31549,31 @@
           <t>WSC330</t>
         </is>
       </c>
-      <c r="E453" s="2" t="inlineStr">
+      <c r="E453" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="F453" s="2" t="inlineStr">
+      <c r="F453" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="G453" s="2" t="n"/>
-      <c r="H453" s="2" t="n"/>
-      <c r="I453" s="2" t="n"/>
-      <c r="J453" s="2" t="n"/>
-      <c r="K453" s="2" t="n"/>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="L453" t="n">
         <v>68.31999999999999</v>
       </c>
@@ -31261,21 +32111,39 @@
           <t>SAF126</t>
         </is>
       </c>
-      <c r="E460" s="2" t="inlineStr">
+      <c r="E460" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="F460" s="2" t="inlineStr">
+      <c r="F460" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="G460" s="2" t="n"/>
-      <c r="H460" s="2" t="n"/>
-      <c r="I460" s="2" t="n"/>
-      <c r="J460" s="2" t="n"/>
-      <c r="K460" s="2" t="n"/>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
+      <c r="J460" t="n">
+        <v>249.9</v>
+      </c>
+      <c r="K460" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="L460" t="n">
         <v>135.3</v>
       </c>
@@ -31750,7 +32618,11 @@
       </c>
       <c r="G466" s="2" t="n"/>
       <c r="H466" s="2" t="n"/>
-      <c r="I466" s="2" t="n"/>
+      <c r="I466" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J466" s="2" t="n"/>
       <c r="K466" s="2" t="n"/>
       <c r="L466" t="n">
@@ -31894,7 +32766,11 @@
       </c>
       <c r="G468" s="2" t="n"/>
       <c r="H468" s="2" t="n"/>
-      <c r="I468" s="2" t="n"/>
+      <c r="I468" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J468" s="2" t="n"/>
       <c r="K468" s="2" t="n"/>
       <c r="L468" t="n">
@@ -32170,7 +33046,11 @@
       </c>
       <c r="G472" s="2" t="n"/>
       <c r="H472" s="2" t="n"/>
-      <c r="I472" s="2" t="n"/>
+      <c r="I472" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J472" s="2" t="n"/>
       <c r="K472" s="2" t="n"/>
       <c r="L472" t="n">
@@ -32233,7 +33113,11 @@
       </c>
       <c r="G473" s="2" t="n"/>
       <c r="H473" s="2" t="n"/>
-      <c r="I473" s="2" t="n"/>
+      <c r="I473" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J473" s="2" t="n"/>
       <c r="K473" s="2" t="n"/>
       <c r="L473" t="n">
@@ -32296,7 +33180,11 @@
       </c>
       <c r="G474" s="2" t="n"/>
       <c r="H474" s="2" t="n"/>
-      <c r="I474" s="2" t="n"/>
+      <c r="I474" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J474" s="2" t="n"/>
       <c r="K474" s="2" t="n"/>
       <c r="L474" t="n">
@@ -32680,7 +33568,11 @@
       </c>
       <c r="G479" s="2" t="n"/>
       <c r="H479" s="2" t="n"/>
-      <c r="I479" s="2" t="n"/>
+      <c r="I479" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J479" s="2" t="n"/>
       <c r="K479" s="2" t="n"/>
       <c r="L479" t="n">
@@ -32743,7 +33635,11 @@
       </c>
       <c r="G480" s="2" t="n"/>
       <c r="H480" s="2" t="n"/>
-      <c r="I480" s="2" t="n"/>
+      <c r="I480" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J480" s="2" t="n"/>
       <c r="K480" s="2" t="n"/>
       <c r="L480" t="n">
@@ -32806,7 +33702,11 @@
       </c>
       <c r="G481" s="2" t="n"/>
       <c r="H481" s="2" t="n"/>
-      <c r="I481" s="2" t="n"/>
+      <c r="I481" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J481" s="2" t="n"/>
       <c r="K481" s="2" t="n"/>
       <c r="L481" t="n">
@@ -33634,7 +34534,11 @@
       </c>
       <c r="G493" s="2" t="n"/>
       <c r="H493" s="2" t="n"/>
-      <c r="I493" s="2" t="n"/>
+      <c r="I493" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J493" s="2" t="n"/>
       <c r="K493" s="2" t="n"/>
       <c r="L493" t="n">
@@ -33682,7 +34586,11 @@
       </c>
       <c r="G494" s="2" t="n"/>
       <c r="H494" s="2" t="n"/>
-      <c r="I494" s="2" t="n"/>
+      <c r="I494" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J494" s="2" t="n"/>
       <c r="K494" s="2" t="n"/>
       <c r="L494" t="n">
@@ -33730,7 +34638,11 @@
       </c>
       <c r="G495" s="2" t="n"/>
       <c r="H495" s="2" t="n"/>
-      <c r="I495" s="2" t="n"/>
+      <c r="I495" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J495" s="2" t="n"/>
       <c r="K495" s="2" t="n"/>
       <c r="L495" t="n">
@@ -33778,7 +34690,11 @@
       </c>
       <c r="G496" s="2" t="n"/>
       <c r="H496" s="2" t="n"/>
-      <c r="I496" s="2" t="n"/>
+      <c r="I496" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J496" s="2" t="n"/>
       <c r="K496" s="2" t="n"/>
       <c r="L496" t="n">
@@ -33826,7 +34742,11 @@
       </c>
       <c r="G497" s="2" t="n"/>
       <c r="H497" s="2" t="n"/>
-      <c r="I497" s="2" t="n"/>
+      <c r="I497" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J497" s="2" t="n"/>
       <c r="K497" s="2" t="n"/>
       <c r="L497" t="n">
@@ -34006,7 +34926,11 @@
       </c>
       <c r="G500" s="2" t="n"/>
       <c r="H500" s="2" t="n"/>
-      <c r="I500" s="2" t="n"/>
+      <c r="I500" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J500" s="2" t="n"/>
       <c r="K500" s="2" t="n"/>
       <c r="L500" t="n">
@@ -34054,7 +34978,11 @@
       </c>
       <c r="G501" s="2" t="n"/>
       <c r="H501" s="2" t="n"/>
-      <c r="I501" s="2" t="n"/>
+      <c r="I501" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J501" s="2" t="n"/>
       <c r="K501" s="2" t="n"/>
       <c r="L501" t="n">
@@ -34102,7 +35030,11 @@
       </c>
       <c r="G502" s="2" t="n"/>
       <c r="H502" s="2" t="n"/>
-      <c r="I502" s="2" t="n"/>
+      <c r="I502" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J502" s="2" t="n"/>
       <c r="K502" s="2" t="n"/>
       <c r="L502" t="n">
@@ -35383,7 +36315,11 @@
       </c>
       <c r="G521" s="2" t="n"/>
       <c r="H521" s="2" t="n"/>
-      <c r="I521" s="2" t="n"/>
+      <c r="I521" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J521" s="2" t="n"/>
       <c r="K521" s="2" t="n"/>
       <c r="L521" t="n">
@@ -35446,7 +36382,11 @@
       </c>
       <c r="G522" s="2" t="n"/>
       <c r="H522" s="2" t="n"/>
-      <c r="I522" s="2" t="n"/>
+      <c r="I522" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J522" s="2" t="n"/>
       <c r="K522" s="2" t="n"/>
       <c r="L522" t="n">
@@ -35509,7 +36449,11 @@
       </c>
       <c r="G523" s="2" t="n"/>
       <c r="H523" s="2" t="n"/>
-      <c r="I523" s="2" t="n"/>
+      <c r="I523" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J523" s="2" t="n"/>
       <c r="K523" s="2" t="n"/>
       <c r="L523" t="n">
@@ -35836,7 +36780,11 @@
       </c>
       <c r="G528" s="2" t="n"/>
       <c r="H528" s="2" t="n"/>
-      <c r="I528" s="2" t="n"/>
+      <c r="I528" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J528" s="2" t="n"/>
       <c r="K528" s="2" t="n"/>
       <c r="L528" t="n">
@@ -35899,7 +36847,11 @@
       </c>
       <c r="G529" s="2" t="n"/>
       <c r="H529" s="2" t="n"/>
-      <c r="I529" s="2" t="n"/>
+      <c r="I529" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J529" s="2" t="n"/>
       <c r="K529" s="2" t="n"/>
       <c r="L529" t="n">
@@ -35962,7 +36914,11 @@
       </c>
       <c r="G530" s="2" t="n"/>
       <c r="H530" s="2" t="n"/>
-      <c r="I530" s="2" t="n"/>
+      <c r="I530" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J530" s="2" t="n"/>
       <c r="K530" s="2" t="n"/>
       <c r="L530" t="n">
@@ -36025,7 +36981,11 @@
       </c>
       <c r="G531" s="2" t="n"/>
       <c r="H531" s="2" t="n"/>
-      <c r="I531" s="2" t="n"/>
+      <c r="I531" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J531" s="2" t="n"/>
       <c r="K531" s="2" t="n"/>
       <c r="L531" t="n">
@@ -36568,7 +37528,11 @@
       </c>
       <c r="G538" s="2" t="n"/>
       <c r="H538" s="2" t="n"/>
-      <c r="I538" s="2" t="n"/>
+      <c r="I538" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J538" s="2" t="n"/>
       <c r="K538" s="2" t="n"/>
       <c r="L538" t="n">
@@ -36631,7 +37595,11 @@
       </c>
       <c r="G539" s="2" t="n"/>
       <c r="H539" s="2" t="n"/>
-      <c r="I539" s="2" t="n"/>
+      <c r="I539" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J539" s="2" t="n"/>
       <c r="K539" s="2" t="n"/>
       <c r="L539" t="n">
@@ -36694,7 +37662,11 @@
       </c>
       <c r="G540" s="2" t="n"/>
       <c r="H540" s="2" t="n"/>
-      <c r="I540" s="2" t="n"/>
+      <c r="I540" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J540" s="2" t="n"/>
       <c r="K540" s="2" t="n"/>
       <c r="L540" t="n">
@@ -37087,7 +38059,11 @@
       </c>
       <c r="G546" s="2" t="n"/>
       <c r="H546" s="2" t="n"/>
-      <c r="I546" s="2" t="n"/>
+      <c r="I546" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J546" s="2" t="n"/>
       <c r="K546" s="2" t="n"/>
       <c r="L546" t="n">
@@ -37231,7 +38207,11 @@
       </c>
       <c r="G548" s="2" t="n"/>
       <c r="H548" s="2" t="n"/>
-      <c r="I548" s="2" t="n"/>
+      <c r="I548" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J548" s="2" t="n"/>
       <c r="K548" s="2" t="n"/>
       <c r="L548" t="n">
@@ -37294,7 +38274,11 @@
       </c>
       <c r="G549" s="2" t="n"/>
       <c r="H549" s="2" t="n"/>
-      <c r="I549" s="2" t="n"/>
+      <c r="I549" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J549" s="2" t="n"/>
       <c r="K549" s="2" t="n"/>
       <c r="L549" t="n">
@@ -37357,7 +38341,11 @@
       </c>
       <c r="G550" s="2" t="n"/>
       <c r="H550" s="2" t="n"/>
-      <c r="I550" s="2" t="n"/>
+      <c r="I550" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J550" s="2" t="n"/>
       <c r="K550" s="2" t="n"/>
       <c r="L550" t="n">
@@ -37498,7 +38486,11 @@
       </c>
       <c r="G552" s="2" t="n"/>
       <c r="H552" s="2" t="n"/>
-      <c r="I552" s="2" t="n"/>
+      <c r="I552" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J552" s="2" t="n"/>
       <c r="K552" s="2" t="n"/>
       <c r="L552" t="n">
@@ -37564,7 +38556,11 @@
       </c>
       <c r="G553" s="2" t="n"/>
       <c r="H553" s="2" t="n"/>
-      <c r="I553" s="2" t="n"/>
+      <c r="I553" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J553" s="2" t="n"/>
       <c r="K553" s="2" t="n"/>
       <c r="L553" t="n">
@@ -37630,7 +38626,11 @@
       </c>
       <c r="G554" s="2" t="n"/>
       <c r="H554" s="2" t="n"/>
-      <c r="I554" s="2" t="n"/>
+      <c r="I554" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J554" s="2" t="n"/>
       <c r="K554" s="2" t="n"/>
       <c r="L554" t="n">
@@ -37696,7 +38696,11 @@
       </c>
       <c r="G555" s="2" t="n"/>
       <c r="H555" s="2" t="n"/>
-      <c r="I555" s="2" t="n"/>
+      <c r="I555" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J555" s="2" t="n"/>
       <c r="K555" s="2" t="n"/>
       <c r="L555" t="n">
@@ -37762,7 +38766,11 @@
       </c>
       <c r="G556" s="2" t="n"/>
       <c r="H556" s="2" t="n"/>
-      <c r="I556" s="2" t="n"/>
+      <c r="I556" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J556" s="2" t="n"/>
       <c r="K556" s="2" t="n"/>
       <c r="L556" t="n">
@@ -37828,7 +38836,11 @@
       </c>
       <c r="G557" s="2" t="n"/>
       <c r="H557" s="2" t="n"/>
-      <c r="I557" s="2" t="n"/>
+      <c r="I557" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J557" s="2" t="n"/>
       <c r="K557" s="2" t="n"/>
       <c r="L557" t="n">
@@ -37894,7 +38906,11 @@
       </c>
       <c r="G558" s="2" t="n"/>
       <c r="H558" s="2" t="n"/>
-      <c r="I558" s="2" t="n"/>
+      <c r="I558" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J558" s="2" t="n"/>
       <c r="K558" s="2" t="n"/>
       <c r="L558" t="n">
@@ -38038,7 +39054,11 @@
       </c>
       <c r="G560" s="2" t="n"/>
       <c r="H560" s="2" t="n"/>
-      <c r="I560" s="2" t="n"/>
+      <c r="I560" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J560" s="2" t="n"/>
       <c r="K560" s="2" t="n"/>
       <c r="L560" t="n">
@@ -38101,7 +39121,11 @@
       </c>
       <c r="G561" s="2" t="n"/>
       <c r="H561" s="2" t="n"/>
-      <c r="I561" s="2" t="n"/>
+      <c r="I561" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J561" s="2" t="n"/>
       <c r="K561" s="2" t="n"/>
       <c r="L561" t="n">
@@ -38164,7 +39188,11 @@
       </c>
       <c r="G562" s="2" t="n"/>
       <c r="H562" s="2" t="n"/>
-      <c r="I562" s="2" t="n"/>
+      <c r="I562" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J562" s="2" t="n"/>
       <c r="K562" s="2" t="n"/>
       <c r="L562" t="n">
@@ -38227,7 +39255,11 @@
       </c>
       <c r="G563" s="2" t="n"/>
       <c r="H563" s="2" t="n"/>
-      <c r="I563" s="2" t="n"/>
+      <c r="I563" s="2" t="inlineStr">
+        <is>
+          <t>Inverno26</t>
+        </is>
+      </c>
       <c r="J563" s="2" t="n"/>
       <c r="K563" s="2" t="n"/>
       <c r="L563" t="n">

</xml_diff>